<commit_message>
SPO and SPP corrections
Corrected and updated some errors/improvements
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026_4sfera_com.xlsx
+++ b/AQD R3 DDBB views 2026_4sfera_com.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\albal\Desktop\AQD Semana 20 al 24\R3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lallana\Desktop\Cambios R3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C068F70C-5EC6-4D7A-8667-708700B2E712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5220EFB-A9F4-4BAF-880C-D3574C18575A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14190" yWindow="0" windowWidth="14610" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6264" yWindow="720" windowWidth="17280" windowHeight="9024" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SamplingProcess (SPP)" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,11 @@
     <sheet name="ZoneGeometry (ZOG)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1390,6 +1395,27 @@
     <t>https://taskman.eionet.europa.eu/issues/305543</t>
   </si>
   <si>
+    <t>[qc].[SPO_01_A]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_02_A]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_02_B]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_02_C]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_02_D]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_03_C]</t>
+  </si>
+  <si>
+    <t>[qc].[SPO_04_B]</t>
+  </si>
+  <si>
     <t>SamplingPointRef</t>
   </si>
   <si>
@@ -1654,80 +1680,59 @@
     <t xml:space="preserve">ZoneGeometry (ZOG) </t>
   </si>
   <si>
+    <t>ZOG_PK</t>
+  </si>
+  <si>
+    <t>The combination of CountryCode (ZOG_01) and ZoneId (ZOG_02) must uniquely identify each record in the ZoneGeometry table and neither attribute may be null.</t>
+  </si>
+  <si>
+    <t>ZOG_0</t>
+  </si>
+  <si>
+    <t>The combination of values reported for the primary key attributes (CountryCode, ZoneId) is checked against the reference ZoneGeometry table. If no matching record exists, the record is classified as 'Addition of new record'. If a matching record exists and zone geometries are identical, the record is classified as 'No modification'. If a matching record exists but zone geometries differ, the record is classified as 'Modification of existing record'.</t>
+  </si>
+  <si>
     <t>ZOG_01_A</t>
   </si>
   <si>
+    <t>Attribute ZOG_01 must correspond to one of the values of Notation in [Airquality_R3].[reference].[Vocabulary] where vocabulary = 'countries'.</t>
+  </si>
+  <si>
     <t>ZOG_02_A</t>
   </si>
   <si>
+    <t>Attribute ZOG_02 must have length &gt; 0 and must be unique within the same CountryCode.</t>
+  </si>
+  <si>
     <t>ZOG_02_B</t>
   </si>
   <si>
-    <t>ZOG_0</t>
-  </si>
-  <si>
-    <t>ZOG_PK</t>
+    <t>Attribute ZOG_02 should follow the recommended naming convention ZON{separator}{CountryCode}, where {separator} is '.', '_' or '-', and {CountryCode} complies with ISO2.</t>
   </si>
   <si>
     <t>ZOG_03_A</t>
   </si>
   <si>
+    <t>Attribute ZOG_03 must contain a valid geometry that can be successfully parsed and must not contain topological errors such as self-intersections, unclosed polygons or invalid rings.</t>
+  </si>
+  <si>
     <t>ZOG_03_B</t>
   </si>
   <si>
+    <t>Attribute ZOG_03 must represent the territory of the reporting CountryCode and must not overlap the land territory of another country.</t>
+  </si>
+  <si>
     <t>ZOG_03_C</t>
   </si>
   <si>
-    <t>The combination of values reported for the primary key attributes (CountryCode, ZoneId) is checked against the reference ZoneGeometry table. If no matching record exists, the record is classified as 'Addition of new record'. If a matching record exists and zone geometries are identical, the record is classified as 'No modification'. If a matching record exists but zone geometries differ, the record is classified as 'Modification of existing record'.</t>
-  </si>
-  <si>
     <t>Attribute ZOG_03 must use one of the supported coordinate reference systems: EPSG:3035, EPSG:4258 or EPSG:4326.</t>
-  </si>
-  <si>
-    <t>Attribute ZOG_03 must represent the territory of the reporting CountryCode and must not overlap the land territory of another country.</t>
-  </si>
-  <si>
-    <t>Attribute ZOG_03 must contain a valid geometry that can be successfully parsed and must not contain topological errors such as self-intersections, unclosed polygons or invalid rings.</t>
-  </si>
-  <si>
-    <t>The combination of CountryCode (ZOG_01) and ZoneId (ZOG_02) must uniquely identify each record in the ZoneGeometry table and neither attribute may be null.</t>
-  </si>
-  <si>
-    <t>Attribute ZOG_01 must correspond to one of the values of Notation in [Airquality_R3].[reference].[Vocabulary] where vocabulary = 'countries'.</t>
-  </si>
-  <si>
-    <t>Attribute ZOG_02 must have length &gt; 0 and must be unique within the same CountryCode.</t>
-  </si>
-  <si>
-    <t>Attribute ZOG_02 should follow the recommended naming convention ZON{separator}{CountryCode}, where {separator} is '.', '_' or '-', and {CountryCode} complies with ISO2.</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_04_B]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_03_C]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_02_D]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_02_C]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_02_B]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_02_A]</t>
-  </si>
-  <si>
-    <t>[qc].[SPO_01_A]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1824,14 +1829,8 @@
       <sz val="9"/>
       <name val="Tahoma"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1852,7 +1851,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -1870,6 +1869,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
@@ -1895,8 +1900,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
@@ -1908,19 +1913,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FA9C"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -1931,12 +1929,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -2007,17 +2011,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2025,23 +2018,27 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2049,8 +2046,9 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2068,7 +2066,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2078,33 +2076,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -2225,11 +2221,6 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFF8FA9C"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2243,24 +2234,24 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="tc={98339C65-A981-4E71-B011-09FFEF030360}" id="{BA9CAD86-DC76-713B-DB69-8ED57EF5A5FD}"/>
-  <person displayName="tc={BC8092FB-ED06-4F30-BB5A-3740F72BE98B}" id="{4EA5EE91-C43C-2A46-CF0F-686386B20E5B}"/>
-  <person displayName="tc={490B77A0-62D5-4524-8722-2821422E9730}" id="{41B4127A-4E5E-99E9-572B-42C660D99634}"/>
-  <person displayName="tc={8FFECDF7-F7B5-415B-895C-2A49C7898D2E}" id="{159912E2-EEF8-75A3-CD60-9421597C7293}"/>
-  <person displayName="tc={30CCE20F-0910-4B3E-B84F-8FCC06678552}" id="{37187DD2-730B-8001-9D41-8B1CE9783956}"/>
-  <person displayName="tc={3DA4E063-7EDE-42C2-89DC-071A89E072CE}" id="{441C331A-C848-EDEF-B658-023AC30C5DB4}"/>
-  <person displayName="tc={3E8DD45C-46E7-465E-8876-4919E45020C6}" id="{15D5DA6D-0535-37B2-F663-385ED6EB15FA}"/>
-  <person displayName="tc={54D61B2D-210B-4D09-86A7-B45CE962A4B8}" id="{2368CFE4-C4D9-1109-F680-218ADD419955}"/>
-  <person displayName="tc={E347F355-D485-4768-9BD7-1A96560682D0}" id="{CE472ABB-99FE-7D2D-E1A0-1065DC798D9D}"/>
-  <person displayName="tc={1E85BB37-0120-43BF-94F4-7A83479F1A4F}" id="{D5EF1333-F505-E3FE-802F-7AE6502E9EE4}"/>
-  <person displayName="tc={A573D4B5-DC98-495C-A577-BD4C21E95BCB}" id="{6BD42DDA-00F7-D9AC-2D3E-3775812FA148}"/>
-  <person displayName="tc={20493F91-5BBC-482C-9C73-D643F028C2D4}" id="{3C21631F-FBE8-5E0F-3931-30AC256F3193}"/>
-  <person displayName="tc={52122516-33F3-4456-8E6E-9B680A5AD7E3}" id="{04A368A1-5DA5-E72B-A214-469A143D7F67}"/>
-  <person displayName="tc={29CB7204-F2B2-4884-8A8B-64AE37F06BE6}" id="{9361552C-F8A0-1A6B-665A-93210D17C8FA}"/>
-  <person displayName="tc={BF0E0883-33BA-43E0-BF35-EC267681D38F}" id="{C8027AD9-261C-3D1C-276F-A4CDC33DE1F1}"/>
-  <person displayName="tc={CF358EB7-C8E0-4BDE-AD85-1E5D278FC4A6}" id="{5F3BF8B5-B341-159C-38E9-AEDD0DA5133E}"/>
-  <person displayName="tc={0A0E88C7-8798-478D-95CD-9D699DD4076D}" id="{D55D8047-0F84-D6AE-5135-A34862A46EF0}"/>
-  <person displayName="tc={680D8D74-A90F-40EB-8152-C2AC5B1BD190}" id="{8DD2AC5C-B1A0-39ED-E72C-1FCF4A1D04C9}"/>
+  <person displayName="tc={98339c65-a981-4e71-b011-09ffef030360}" id="{2FFCC802-290F-A181-67E9-9C1FB06B16B7}"/>
+  <person displayName="tc={bc8092fb-ed06-4f30-bb5a-3740f72be98b}" id="{3B10C98B-12F6-CEA5-663B-22D5674EBE2A}"/>
+  <person displayName="tc={490b77a0-62d5-4524-8722-2821422e9730}" id="{1B31B7B1-7F12-2A29-CFB1-49CF8E7C8D1B}"/>
+  <person displayName="tc={8ffecdf7-f7b5-415b-895c-2a49c7898d2e}" id="{4BA197E0-565D-B4CD-48F6-892443E0FE5A}"/>
+  <person displayName="tc={30cce20f-0910-4b3e-b84f-8fcc06678552}" id="{4533ACC3-D2D9-421D-E2D9-DD5BBC954281}"/>
+  <person displayName="tc={3da4e063-7ede-42c2-89dc-071a89e072ce}" id="{B86E3BCE-DB44-F70C-4F19-A905D2C6DA35}"/>
+  <person displayName="tc={3e8dd45c-46e7-465e-8876-4919e45020c6}" id="{C5B26D5A-1FAB-CCEB-1798-409D1CA99359}"/>
+  <person displayName="tc={54d61b2d-210b-4d09-86a7-b45ce962a4b8}" id="{B357EAE8-074C-556E-B445-E557AC811191}"/>
+  <person displayName="tc={e347f355-d485-4768-9bd7-1a96560682d0}" id="{A2E2009C-EA6B-4971-F6E3-5A907E3C75EF}"/>
+  <person displayName="tc={1e85bb37-0120-43bf-94f4-7a83479f1a4f}" id="{90F399EE-5AD3-4BB5-4CB3-5AC18E1730C2}"/>
+  <person displayName="tc={a573d4b5-dc98-495c-a577-bd4c21e95bcb}" id="{213A65BA-8F48-8AFF-71F5-22CCA5765ACD}"/>
+  <person displayName="tc={20493f91-5bbc-482c-9c73-d643f028c2d4}" id="{9E5FF495-DF5E-8E27-8D51-71042DA4EE85}"/>
+  <person displayName="tc={52122516-33f3-4456-8e6e-9b680a5ad7e3}" id="{2C5FE0D2-EA13-B987-FA4A-10E40558B40F}"/>
+  <person displayName="tc={29cb7204-f2b2-4884-8a8b-64ae37f06be6}" id="{83940ACE-E867-47D2-FC2B-B9DC6DDE3EB5}"/>
+  <person displayName="tc={bf0e0883-33ba-43e0-bf35-ec267681d38f}" id="{C98B2C38-5018-19BA-51C9-F28AAF6A12C7}"/>
+  <person displayName="tc={cf358eb7-c8e0-4bde-ad85-1e5d278fc4a6}" id="{4566558B-34AE-FCD8-B670-0A7AB2298808}"/>
+  <person displayName="tc={0a0e88c7-8798-478d-95cd-9d699dd4076d}" id="{34F2EA13-14CC-C373-F261-EBD239A18C63}"/>
+  <person displayName="tc={680d8d74-a90f-40eb-8152-c2ac5b1bd190}" id="{1E054922-84FC-8C7E-BDBC-C675B6FCA1B2}"/>
 </personList>
 </file>
 
@@ -2283,11 +2274,11 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{66ABB4FB-5285-49AE-9464-AEF282784317}" name="Table911" displayName="Table911" ref="A17:B18">
-  <autoFilter ref="A17:B18" xr:uid="{66ABB4FB-5285-49AE-9464-AEF282784317}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Table911" displayName="Table911" ref="A17:B18">
+  <autoFilter ref="A17:B18" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{0B5475EE-A748-44D7-A365-9BE8888D5DA0}" name="OLD name"/>
-    <tableColumn id="2" xr3:uid="{7608104F-4AEF-48B1-A43B-392CACD0807C}" name="NEW name"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="OLD name"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="NEW name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2392,18 +2383,18 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A7563493-AFB1-4A5A-8B6A-D7659AEDA3EA}" name="Table134710" displayName="Table134710" ref="A2:I10">
-  <autoFilter ref="A2:I10" xr:uid="{A7563493-AFB1-4A5A-8B6A-D7659AEDA3EA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Table134710" displayName="Table134710" ref="A2:I10">
+  <autoFilter ref="A2:I10" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{7B4FB171-7024-4F09-B41F-120549610F4B}" name="Table"/>
-    <tableColumn id="2" xr3:uid="{F502886B-DE51-4397-B79E-94315A2D8D16}" name="QC rule" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{5D808FF7-11A3-40C4-AB75-5538989DDCF4}" name="Description" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{C15BFA07-7901-454E-9609-71F2ABD591FF}" name="Task" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{66FF3DD9-3747-4DDC-8338-2AC1165D7630}" name="Task 2" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{36E72C8C-0507-4BFD-9F9D-CC9A0C5ACB4D}" name="Status" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{65FD5A7C-426B-42C8-AA05-79F082BD9EB7}" name="Github" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{309C54B1-66E3-40B1-B65A-008E6561A080}" name="Tested" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{C2DAD112-80A4-4982-B7DC-96FE683D5323}" name="Comments" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Table"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="QC rule"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Description"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Task"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Task 2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="Status"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Github"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="Tested"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2627,15 +2618,15 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B21" dT="2026-07-08T07:18:15.56Z" personId="{ba9cad86-dc76-713b-db69-8ed57ef5a5fd}" id="{98339c65-a981-4e71-b011-09ffef030360}" done="0">
+  <threadedComment ref="B21" dT="2026-07-08T07:18:15.56Z" personId="{2ffcc802-290f-a181-67e9-9c1fb06b16b7}" id="{98339c65-a981-4e71-b011-09ffef030360}" done="0">
     <text xml:space="preserve">Is this needed??? We have 07_A and we check if appears int he Vocabulary Table
 </text>
   </threadedComment>
-  <threadedComment ref="B24" dT="2026-07-08T08:38:26.82Z" personId="{4ea5ee91-c43c-2a46-cf0f-686386b20e5b}" id="{bc8092fb-ed06-4f30-bb5a-3740f72be98b}" done="0">
+  <threadedComment ref="B24" dT="2026-07-08T08:38:26.82Z" personId="{3b10c98b-12f6-cea5-663b-22d5674ebe2a}" id="{bc8092fb-ed06-4f30-bb5a-3740f72be98b}" done="0">
     <text xml:space="preserve">I should replace this QA with two different QAs. 
 </text>
   </threadedComment>
-  <threadedComment ref="B9" dT="2026-07-08T08:39:09.89Z" personId="{41b4127a-4e5e-99e9-572b-42c660d99634}" id="{490b77a0-62d5-4524-8722-2821422e9730}" done="0">
+  <threadedComment ref="B9" dT="2026-07-08T08:39:09.89Z" personId="{1b31b7b1-7f12-2a29-cfb1-49cf8e7c8d1b}" id="{490b77a0-62d5-4524-8722-2821422e9730}" done="0">
     <text xml:space="preserve">I should replace this QA with two different QAs. 
 </text>
   </threadedComment>
@@ -2644,15 +2635,15 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B12" dT="2026-07-07T11:47:46.10Z" personId="{159912e2-eef8-75a3-cd60-9421597c7293}" id="{8ffecdf7-f7b5-415b-895c-2a49c7898d2e}" done="0">
+  <threadedComment ref="B12" dT="2026-07-07T11:47:46.10Z" personId="{4ba197e0-565d-b4cd-48f6-892443e0fe5a}" id="{8ffecdf7-f7b5-415b-895c-2a49c7898d2e}" done="0">
     <text xml:space="preserve">I should replace this QA with two different QAs. 
 </text>
   </threadedComment>
-  <threadedComment ref="B14" dT="2026-07-07T11:53:25.68Z" personId="{37187dd2-730b-8001-9d41-8b1ce9783956}" id="{30cce20f-0910-4b3e-b84f-8fcc06678552}" done="0">
+  <threadedComment ref="B14" dT="2026-07-07T11:53:25.68Z" personId="{4533acc3-d2d9-421d-e2d9-dd5bbc954281}" id="{30cce20f-0910-4b3e-b84f-8fcc06678552}" done="0">
     <text xml:space="preserve">I think it’s necessary to create more QCs for this attribute
 </text>
   </threadedComment>
-  <threadedComment ref="B7" dT="2026-07-07T11:37:08.34Z" personId="{441c331a-c848-edef-b658-023ac30c5db4}" id="{3da4e063-7ede-42c2-89dc-071a89e072ce}" done="0">
+  <threadedComment ref="B7" dT="2026-07-07T11:37:08.34Z" personId="{b86e3bce-db44-f70c-4f19-a905d2c6da35}" id="{3da4e063-7ede-42c2-89dc-071a89e072ce}" done="0">
     <text xml:space="preserve">I think this QA is not correct. See “STA_07_A should be testing StationNationalCode (StationEoICode is tested in STA_02_ QC rules)” (see STA_02_B new)
 </text>
   </threadedComment>
@@ -2661,23 +2652,23 @@
 
 <file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B3" dT="2026-07-07T12:24:03.07Z" personId="{15d5da6d-0535-37b2-f663-385ed6eb15fa}" id="{3e8dd45c-46e7-465e-8876-4919e45020c6}" done="0">
+  <threadedComment ref="B3" dT="2026-07-07T12:24:03.07Z" personId="{c5b26d5a-1fab-cceb-1798-409d1ca99359}" id="{3e8dd45c-46e7-465e-8876-4919e45020c6}" done="0">
     <text xml:space="preserve">It should be renamed as SPO_04_A because PollutantId is SPO_04
 </text>
   </threadedComment>
-  <threadedComment ref="B4" dT="2026-07-07T12:34:08.20Z" personId="{2368cfe4-c4d9-1109-f680-218add419955}" id="{54d61b2d-210b-4d09-86a7-b45ce962a4b8}" done="0">
+  <threadedComment ref="B4" dT="2026-07-07T12:34:08.20Z" personId="{b357eae8-074c-556e-b445-e557ac811191}" id="{54d61b2d-210b-4d09-86a7-b45ce962a4b8}" done="0">
     <text xml:space="preserve">It should be renamed as SPO_04_B because PollutantId is SPO_04
 </text>
   </threadedComment>
-  <threadedComment ref="B5" dT="2026-07-08T06:08:12.99Z" personId="{ce472abb-99fe-7d2d-e1a0-1065dc798d9d}" id="{e347f355-d485-4768-9bd7-1a96560682d0}" done="0">
+  <threadedComment ref="B5" dT="2026-07-08T06:08:12.99Z" personId="{a2e2009c-ea6b-4971-f6e3-5a907e3c75ef}" id="{e347f355-d485-4768-9bd7-1a96560682d0}" done="0">
     <text xml:space="preserve">It should be renamed as SPO_05_A because StationEoICode is SPO_05
 </text>
   </threadedComment>
-  <threadedComment ref="B7" dT="2026-07-07T12:20:54.40Z" personId="{d5ef1333-f505-e3fe-802f-7ae6502e9ee4}" id="{1e85bb37-0120-43bf-94f4-7a83479f1a4f}" done="0">
+  <threadedComment ref="B7" dT="2026-07-07T12:20:54.40Z" personId="{90f399ee-5ad3-4bb5-4cb3-5ac18e1730c2}" id="{1e85bb37-0120-43bf-94f4-7a83479f1a4f}" done="0">
     <text xml:space="preserve">AirQualityStationArea has been moved to SPL
 </text>
   </threadedComment>
-  <threadedComment ref="B8" dT="2026-07-07T12:20:59.37Z" personId="{6bd42dda-00f7-d9ac-2d3e-3775812fa148}" id="{a573d4b5-dc98-495c-a577-bd4c21e95bcb}" done="0">
+  <threadedComment ref="B8" dT="2026-07-07T12:20:59.37Z" personId="{213a65ba-8f48-8aff-71f5-22cca5765acd}" id="{a573d4b5-dc98-495c-a577-bd4c21e95bcb}" done="0">
     <text xml:space="preserve">AirQualityStationArea has been moved to SPL
 </text>
   </threadedComment>
@@ -2686,31 +2677,31 @@
 
 <file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B18" dT="2026-07-08T06:27:09.26Z" personId="{3c21631f-fbe8-5e0f-3931-30ac256f3193}" id="{20493f91-5bbc-482c-9c73-d643f028c2d4}" done="0">
+  <threadedComment ref="B18" dT="2026-07-08T06:27:09.26Z" personId="{9e5ff495-df5e-8e27-8d51-71042da4ee85}" id="{20493f91-5bbc-482c-9c73-d643f028c2d4}" done="0">
     <text xml:space="preserve">We propose to merge both QA.
 </text>
   </threadedComment>
-  <threadedComment ref="B20" dT="2026-07-08T06:27:18.69Z" personId="{04a368a1-5da5-e72b-a214-469a143d7f67}" id="{52122516-33f3-4456-8e6e-9b680a5ad7e3}" done="0">
+  <threadedComment ref="B20" dT="2026-07-08T06:27:18.69Z" personId="{2c5fe0d2-ea13-b987-fa4a-10e40558b40f}" id="{52122516-33f3-4456-8e6e-9b680a5ad7e3}" done="0">
     <text xml:space="preserve">We propose to merge both QA.
 </text>
   </threadedComment>
-  <threadedComment ref="B22" dT="2026-07-08T06:30:12.04Z" personId="{9361552c-f8a0-1a6b-665a-93210d17c8fa}" id="{29cb7204-f2b2-4884-8a8b-64ae37f06be6}" done="0">
+  <threadedComment ref="B22" dT="2026-07-08T06:30:12.04Z" personId="{83940ace-e867-47d2-fc2b-b9dc6dde3eb5}" id="{29cb7204-f2b2-4884-8a8b-64ae37f06be6}" done="0">
     <text xml:space="preserve">Now we have -10 and 5700
 </text>
   </threadedComment>
-  <threadedComment ref="B23" dT="2026-07-08T06:31:17.86Z" personId="{c8027ad9-261c-3d1c-276f-a4cdc33de1f1}" id="{bf0e0883-33ba-43e0-bf35-ec267681d38f}" done="0">
+  <threadedComment ref="B23" dT="2026-07-08T06:31:17.86Z" personId="{c98b2c38-5018-19ba-51c9-f28aaf6a12c7}" id="{bf0e0883-33ba-43e0-bf35-ec267681d38f}" done="0">
     <text xml:space="preserve">In the current QA we have 0-30 meters
 </text>
   </threadedComment>
-  <threadedComment ref="B24" dT="2026-07-08T06:43:57.31Z" personId="{5f3bf8b5-b341-159c-38e9-aedd0da5133e}" id="{cf358eb7-c8e0-4bde-ad85-1e5d278fc4a6}" done="0">
+  <threadedComment ref="B24" dT="2026-07-08T06:43:57.31Z" personId="{4566558b-34ae-fcd8-b670-0a7ab2298808}" id="{cf358eb7-c8e0-4bde-ad85-1e5d278fc4a6}" done="0">
     <text xml:space="preserve">It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
 </text>
   </threadedComment>
-  <threadedComment ref="B25" dT="2026-07-08T06:44:12.64Z" personId="{d55d8047-0f84-d6ae-5135-a34862a46ef0}" id="{0a0e88c7-8798-478d-95cd-9d699dd4076d}" done="0">
+  <threadedComment ref="B25" dT="2026-07-08T06:44:12.64Z" personId="{34f2ea13-14cc-c373-f261-ebd239a18c63}" id="{0a0e88c7-8798-478d-95cd-9d699dd4076d}" done="0">
     <text xml:space="preserve">Mandatory SamplingPointCategory = Traffic
 </text>
   </threadedComment>
-  <threadedComment ref="B26" dT="2026-07-08T06:44:58.31Z" personId="{8dd2ac5c-b1a0-39ed-e72c-1fcf4a1d04c9}" id="{680d8d74-a90f-40eb-8152-c2ac5b1bd190}" done="0">
+  <threadedComment ref="B26" dT="2026-07-08T06:44:58.31Z" personId="{1e054922-84fc-8c7e-bdbc-c675b6fca1b2}" id="{680d8d74-a90f-40eb-8152-c2ac5b1bd190}" done="0">
     <text xml:space="preserve">It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
 </text>
   </threadedComment>
@@ -2720,19 +2711,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.09765625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="104" customWidth="1"/>
-    <col min="4" max="4" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.85546875" customWidth="1"/>
+    <col min="4" max="4" width="52.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.8984375" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="8" width="13.42578125" customWidth="1"/>
-    <col min="9" max="9" width="71.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.3984375" customWidth="1"/>
+    <col min="9" max="9" width="71.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2740,7 +2731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2769,7 +2760,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="16.8">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2792,7 +2783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -2818,7 +2809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2844,7 +2835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2870,76 +2861,76 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="43" t="s">
+    <row r="7" spans="1:9" s="3" customFormat="1">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="56" t="s">
+      <c r="F7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="43" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="43" t="b">
+      <c r="G7" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+    <row r="8" spans="1:9" s="3" customFormat="1">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="43" t="s">
+      <c r="C8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="56" t="s">
+      <c r="F8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="43" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="43" t="b">
+      <c r="G8" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="43" t="s">
+    <row r="9" spans="1:9" s="3" customFormat="1">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="43" t="s">
+      <c r="F9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="43" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="43" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G9" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2952,7 +2943,7 @@
       <c r="D10" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F10" t="s">
@@ -2965,7 +2956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -2975,10 +2966,10 @@
       <c r="C11" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>49</v>
       </c>
       <c r="F11" t="s">
@@ -2991,7 +2982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -3004,7 +2995,7 @@
       <c r="D12" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>54</v>
       </c>
       <c r="F12" t="s">
@@ -3017,7 +3008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -3030,7 +3021,7 @@
       <c r="D13" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F13" t="s">
@@ -3043,7 +3034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -3056,7 +3047,7 @@
       <c r="D14" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>62</v>
       </c>
       <c r="F14" t="s">
@@ -3069,7 +3060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -3082,7 +3073,7 @@
       <c r="D15" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>66</v>
       </c>
       <c r="F15" t="s">
@@ -3095,7 +3086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -3108,7 +3099,7 @@
       <c r="D16" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>70</v>
       </c>
       <c r="F16" t="s">
@@ -3121,7 +3112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -3134,7 +3125,7 @@
       <c r="D17" t="s">
         <v>73</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="6" t="s">
         <v>74</v>
       </c>
       <c r="F17" t="s">
@@ -3150,7 +3141,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -3163,7 +3154,7 @@
       <c r="D18" t="s">
         <v>78</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="6" t="s">
         <v>79</v>
       </c>
       <c r="F18" t="s">
@@ -3179,7 +3170,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -3192,7 +3183,7 @@
       <c r="D19" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="6" t="s">
         <v>83</v>
       </c>
       <c r="F19" t="s">
@@ -3205,7 +3196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -3218,7 +3209,7 @@
       <c r="D20" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>87</v>
       </c>
       <c r="F20" t="s">
@@ -3231,20 +3222,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:9">
+      <c r="A21" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E21" s="6"/>
+      <c r="E21" s="8"/>
       <c r="F21" t="s">
         <v>50</v>
       </c>
@@ -3255,43 +3246,43 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
+    <row r="22" spans="1:9" s="3" customFormat="1">
+      <c r="A22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="56" t="s">
+      <c r="B22" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="43" t="s">
+      <c r="C22" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F22" s="56" t="s">
+      <c r="F22" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="43" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="43" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="G22" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="7"/>
       <c r="F23" t="s">
         <v>50</v>
       </c>
@@ -3302,20 +3293,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:9">
+      <c r="A24" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="3"/>
+      <c r="E24" s="7"/>
       <c r="F24" t="s">
         <v>50</v>
       </c>
@@ -3326,136 +3317,136 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+    <row r="25" spans="1:9">
+      <c r="A25" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="D25" s="7"/>
-      <c r="E25" s="8" t="s">
+      <c r="D25" s="10"/>
+      <c r="E25" s="11" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+    <row r="26" spans="1:9" ht="15.6">
+      <c r="A26" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D26" s="7"/>
-      <c r="E26" s="8" t="s">
+      <c r="D26" s="10"/>
+      <c r="E26" s="11" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+    <row r="27" spans="1:9">
+      <c r="A27" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="7"/>
-      <c r="E27" s="8" t="s">
+      <c r="D27" s="10"/>
+      <c r="E27" s="11" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="43" t="s">
+    <row r="28" spans="1:9" s="59" customFormat="1">
+      <c r="A28" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="43" t="s">
+      <c r="B28" s="59" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="43" t="s">
+      <c r="C28" s="59" t="s">
         <v>109</v>
       </c>
-      <c r="E28" s="44" t="s">
+      <c r="E28" s="60" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="43" t="s">
+    <row r="29" spans="1:9" s="59" customFormat="1">
+      <c r="A29" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="43" t="s">
+      <c r="B29" s="59" t="s">
         <v>111</v>
       </c>
-      <c r="C29" s="43" t="s">
+      <c r="C29" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="E29" s="44" t="s">
+      <c r="E29" s="60" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="43" t="s">
+    <row r="30" spans="1:9" s="59" customFormat="1">
+      <c r="A30" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B30" s="43" t="s">
+      <c r="B30" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="C30" s="43" t="s">
+      <c r="C30" s="59" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="44" t="s">
+      <c r="E30" s="60" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="43" t="s">
+    <row r="31" spans="1:9" s="59" customFormat="1">
+      <c r="A31" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B31" s="43" t="s">
+      <c r="B31" s="59" t="s">
         <v>116</v>
       </c>
-      <c r="C31" s="43" t="s">
+      <c r="C31" s="59" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="44" t="s">
+      <c r="E31" s="60" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="43" t="s">
+    <row r="32" spans="1:9" s="59" customFormat="1">
+      <c r="A32" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="43" t="s">
+      <c r="C32" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="E32" s="44" t="s">
+      <c r="E32" s="60" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="43" t="s">
+    <row r="33" spans="1:5" s="59" customFormat="1">
+      <c r="A33" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="43" t="s">
+      <c r="B33" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C33" s="43" t="s">
+      <c r="C33" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="E33" s="44" t="s">
+      <c r="E33" s="60" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
         <v>124</v>
       </c>
@@ -3463,7 +3454,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>126</v>
       </c>
@@ -3471,7 +3462,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
         <v>128</v>
       </c>
@@ -3479,7 +3470,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
         <v>130</v>
       </c>
@@ -3487,7 +3478,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
         <v>131</v>
       </c>
@@ -3495,7 +3486,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5">
       <c r="A40" t="s">
         <v>132</v>
       </c>
@@ -3503,19 +3494,19 @@
         <v>133</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5">
       <c r="A41" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5">
       <c r="A42" t="s">
         <v>135</v>
       </c>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+    </row>
+    <row r="43" spans="1:5">
       <c r="A43" t="s">
         <v>136</v>
       </c>
@@ -3523,7 +3514,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5">
       <c r="A44" t="s">
         <v>138</v>
       </c>
@@ -3531,49 +3522,49 @@
         <v>139</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5">
       <c r="A45" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="10"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="11" t="s">
+    <row r="46" spans="1:5">
+      <c r="A46" s="14"/>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="15" t="s">
         <v>63</v>
       </c>
       <c r="B48" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="12" t="s">
+    <row r="49" spans="1:3">
+      <c r="A49" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="17" t="s">
         <v>94</v>
       </c>
       <c r="C49" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="11" t="s">
+    <row r="50" spans="1:3">
+      <c r="A50" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="16" t="s">
         <v>142</v>
       </c>
       <c r="C50" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="12" t="s">
+    <row r="51" spans="1:3">
+      <c r="A51" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="16" t="s">
         <v>142</v>
       </c>
       <c r="C51" t="s">
@@ -3620,19 +3611,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" customWidth="1"/>
-    <col min="3" max="3" width="102.42578125" customWidth="1"/>
-    <col min="4" max="4" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.85546875" customWidth="1"/>
-    <col min="6" max="6" width="47.140625" customWidth="1"/>
-    <col min="7" max="8" width="13.42578125" customWidth="1"/>
-    <col min="9" max="9" width="185.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.09765625" customWidth="1"/>
+    <col min="3" max="3" width="102.3984375" customWidth="1"/>
+    <col min="4" max="4" width="52.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.8984375" customWidth="1"/>
+    <col min="6" max="6" width="47.09765625" customWidth="1"/>
+    <col min="7" max="8" width="13.3984375" customWidth="1"/>
+    <col min="9" max="9" width="185.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3640,7 +3631,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -3669,20 +3660,20 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="15" customHeight="1">
       <c r="A3" t="s">
         <v>145</v>
       </c>
       <c r="B3" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="19" t="s">
         <v>149</v>
       </c>
       <c r="F3" t="s">
@@ -3694,24 +3685,24 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="20" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>145</v>
       </c>
       <c r="B4" t="s">
         <v>152</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="21" t="s">
         <v>153</v>
       </c>
       <c r="D4" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="22" t="s">
         <v>155</v>
       </c>
       <c r="F4" t="s">
@@ -3724,17 +3715,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>145</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -3750,70 +3741,70 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+    <row r="6" spans="1:9" s="23" customFormat="1">
+      <c r="A6" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="G6" s="19" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="19" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="G6" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="25" customFormat="1">
+      <c r="A7" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="E7" s="21"/>
-      <c r="F7" s="4" t="s">
+      <c r="E7" s="26"/>
+      <c r="F7" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="G7" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="4" t="s">
+      <c r="G7" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="25" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>145</v>
       </c>
       <c r="B8" t="s">
         <v>171</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="21" t="s">
         <v>13</v>
       </c>
       <c r="D8" t="s">
         <v>172</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="22" t="s">
         <v>173</v>
       </c>
       <c r="F8" t="s">
@@ -3826,17 +3817,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>145</v>
       </c>
       <c r="B9" t="s">
         <v>175</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>168</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -3852,23 +3843,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>145</v>
       </c>
       <c r="B10" t="s">
         <v>179</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="13" t="s">
         <v>50</v>
       </c>
       <c r="G10" t="b">
@@ -3881,23 +3872,23 @@
         <v>182</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>145</v>
       </c>
       <c r="B11" t="s">
         <v>183</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="21" t="s">
         <v>184</v>
       </c>
       <c r="D11" t="s">
         <v>185</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="13" t="s">
         <v>50</v>
       </c>
       <c r="G11" t="b">
@@ -3910,34 +3901,34 @@
         <v>187</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:9">
+      <c r="A12" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="27" t="s">
         <v>189</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="23" t="s">
+      <c r="E12" s="7"/>
+      <c r="F12" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="3" t="s">
+      <c r="G12" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>145</v>
       </c>
@@ -3947,13 +3938,13 @@
       <c r="C13" t="s">
         <v>193</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>194</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="13" t="s">
         <v>50</v>
       </c>
       <c r="G13" t="b">
@@ -3966,184 +3957,184 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:9">
+      <c r="A14" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="23" t="s">
+      <c r="E14" s="8"/>
+      <c r="F14" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="G14" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" spans="1:9" ht="27.6">
+      <c r="A15" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="30" t="s">
         <v>200</v>
       </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="26" t="s">
+      <c r="D15" s="11"/>
+      <c r="E15" s="31" t="s">
         <v>201</v>
       </c>
-      <c r="F15" s="27"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-    </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="F15" s="32"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+    </row>
+    <row r="16" spans="1:9" ht="27.6">
+      <c r="A16" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="30" t="s">
         <v>203</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="26" t="s">
+      <c r="D16" s="11"/>
+      <c r="E16" s="31" t="s">
         <v>204</v>
       </c>
-      <c r="F16" s="27"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="28" t="s">
+      <c r="F16" s="32"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="30" t="s">
         <v>206</v>
       </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="26" t="s">
+      <c r="D17" s="11"/>
+      <c r="E17" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="F17" s="27"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-    </row>
-    <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="29" t="s">
+      <c r="F17" s="32"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+    </row>
+    <row r="18" spans="1:9" ht="18" customHeight="1">
+      <c r="A18" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="C18" s="30" t="s">
+      <c r="C18" s="35" t="s">
         <v>209</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="26" t="s">
+      <c r="D18" s="11"/>
+      <c r="E18" s="31" t="s">
         <v>210</v>
       </c>
-      <c r="F18" s="27"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
+      <c r="F18" s="32"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+    </row>
+    <row r="19" spans="1:9" ht="27.6">
+      <c r="A19" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C19" s="35" t="s">
         <v>212</v>
       </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="26" t="s">
+      <c r="D19" s="11"/>
+      <c r="E19" s="31" t="s">
         <v>213</v>
       </c>
-      <c r="F19" s="27"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-    </row>
-    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
+      <c r="F19" s="32"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="D20" s="8"/>
-      <c r="E20" s="26" t="s">
+      <c r="D20" s="11"/>
+      <c r="E20" s="31" t="s">
         <v>216</v>
       </c>
-      <c r="F20" s="27"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-    </row>
-    <row r="21" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="F20" s="32"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+    </row>
+    <row r="21" spans="1:9" ht="13.5" customHeight="1">
+      <c r="A21" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="30" t="s">
         <v>217</v>
       </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="26" t="s">
+      <c r="D21" s="11"/>
+      <c r="E21" s="31" t="s">
         <v>218</v>
       </c>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+    </row>
+    <row r="22" spans="1:9" ht="27.6">
+      <c r="A22" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="C22" s="30" t="s">
         <v>220</v>
       </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="26" t="s">
+      <c r="D22" s="11"/>
+      <c r="E22" s="31" t="s">
         <v>221</v>
       </c>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>124</v>
       </c>
@@ -4151,7 +4142,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>222</v>
       </c>
@@ -4159,7 +4150,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>224</v>
       </c>
@@ -4167,7 +4158,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>132</v>
       </c>
@@ -4175,7 +4166,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>227</v>
       </c>
@@ -4183,53 +4174,53 @@
         <v>228</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="16"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" s="31"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" s="32"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" s="33"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="31"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="31"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" s="32"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" s="33"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" s="31"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" s="31"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="32"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" s="33"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" s="31"/>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" s="31"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="32"/>
+    <row r="34" spans="1:1">
+      <c r="A34" s="20"/>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="36"/>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" s="36"/>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="37"/>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="38"/>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="36"/>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="36"/>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="37"/>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="38"/>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="36"/>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="36"/>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="37"/>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="38"/>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="36"/>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="36"/>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="37"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4269,18 +4260,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.59765625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="82.42578125" customWidth="1"/>
+    <col min="3" max="3" width="82.3984375" customWidth="1"/>
     <col min="4" max="4" width="45" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="54.28515625" customWidth="1"/>
-    <col min="9" max="9" width="109.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.296875" customWidth="1"/>
+    <col min="9" max="9" width="109.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4288,7 +4279,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4317,90 +4308,90 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:9" ht="16.8">
+      <c r="A3" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="7" t="s">
         <v>234</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="G3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="3" t="s">
+      <c r="G3" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:9" ht="16.8">
+      <c r="A4" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="39" t="s">
         <v>239</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="7" t="s">
         <v>240</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="G4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="G4" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="8" t="s">
         <v>244</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="G5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" ht="90.75" x14ac:dyDescent="0.3">
+      <c r="G5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="7"/>
+    </row>
+    <row r="6" spans="1:9" ht="70.8">
       <c r="A6" t="s">
         <v>231</v>
       </c>
@@ -4410,10 +4401,10 @@
       <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="F6" s="35" t="s">
+      <c r="F6" s="40" t="s">
         <v>249</v>
       </c>
       <c r="G6" t="b">
@@ -4423,21 +4414,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:9" ht="16.8">
+      <c r="A7" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="39" t="s">
         <v>251</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="36" t="s">
+      <c r="E7" s="7"/>
+      <c r="F7" s="41" t="s">
         <v>253</v>
       </c>
       <c r="G7" t="b">
@@ -4446,25 +4437,25 @@
       <c r="H7" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="36" t="s">
+      <c r="I7" s="41" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:9" ht="16.8">
+      <c r="A8" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="39" t="s">
         <v>256</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="36" t="s">
+      <c r="E8" s="7"/>
+      <c r="F8" s="41" t="s">
         <v>253</v>
       </c>
       <c r="G8" t="b">
@@ -4473,11 +4464,11 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="36" t="s">
+      <c r="I8" s="41" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="16.8">
       <c r="A9" t="s">
         <v>231</v>
       </c>
@@ -4487,7 +4478,7 @@
       <c r="C9" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>260</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -4506,215 +4497,215 @@
         <v>263</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:9">
+      <c r="A10" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="30" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7" t="s">
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="25"/>
-    </row>
-    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="F10" s="30"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="30"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7" t="s">
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="25"/>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="F11" s="30"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="30"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="30" t="s">
         <v>270</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7" t="s">
+      <c r="D12" s="10"/>
+      <c r="E12" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="F12" s="25"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="25"/>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="F12" s="30"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="30"/>
+    </row>
+    <row r="13" spans="1:9" ht="41.4">
+      <c r="A13" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7" t="s">
+      <c r="D13" s="10"/>
+      <c r="E13" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="F13" s="25"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="25"/>
-    </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="F13" s="30"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="30"/>
+    </row>
+    <row r="14" spans="1:9" ht="27.6">
+      <c r="A14" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7" t="s">
+      <c r="D14" s="10"/>
+      <c r="E14" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="25"/>
-    </row>
-    <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="F14" s="30"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="30"/>
+    </row>
+    <row r="15" spans="1:9" ht="16.8">
       <c r="C15" s="1"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="37"/>
-    </row>
-    <row r="16" spans="1:9" s="43" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A16" s="51" t="s">
+      <c r="D15" s="6"/>
+      <c r="E15" s="42"/>
+    </row>
+    <row r="16" spans="1:9" s="3" customFormat="1" ht="16.8">
+      <c r="A16" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C16" s="52" t="s">
+      <c r="C16" s="44" t="s">
         <v>259</v>
       </c>
-      <c r="D16" s="53" t="s">
+      <c r="D16" s="45" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="42" t="s">
+    <row r="17" spans="1:2">
+      <c r="A17" s="46" t="s">
         <v>231</v>
       </c>
       <c r="B17" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="51" t="s">
+    <row r="18" spans="1:2" s="3" customFormat="1">
+      <c r="A18" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B18" s="43" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="51" t="s">
+      <c r="B18" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="3" customFormat="1">
+      <c r="A19" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B19" s="43" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="51" t="s">
+      <c r="B19" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="3" customFormat="1">
+      <c r="A20" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B20" s="43" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="51" t="s">
+      <c r="B20" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" s="3" customFormat="1">
+      <c r="A21" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B21" s="43" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="51" t="s">
+      <c r="B21" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="3" customFormat="1">
+      <c r="A22" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B22" s="43" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="51" t="s">
+      <c r="B22" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" s="3" customFormat="1">
+      <c r="A23" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B23" s="43" t="s">
+      <c r="B23" s="3" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="55" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="54" t="s">
+    <row r="24" spans="1:2" s="47" customFormat="1">
+      <c r="A24" s="48" t="s">
         <v>231</v>
       </c>
-      <c r="B24" s="55" t="s">
+      <c r="B24" s="47" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="25" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="51" t="s">
+    <row r="25" spans="1:2" s="3" customFormat="1">
+      <c r="A25" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B25" s="43" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="51" t="s">
+      <c r="B25" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" s="3" customFormat="1">
+      <c r="A26" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="3" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="27" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="51" t="s">
+    <row r="27" spans="1:2" s="3" customFormat="1">
+      <c r="A27" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="B27" s="43" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="51"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="42"/>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" s="3" customFormat="1">
+      <c r="A28" s="43"/>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="46"/>
+    </row>
+    <row r="35" spans="1:2">
       <c r="A35" t="s">
         <v>124</v>
       </c>
@@ -4722,7 +4713,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" t="s">
         <v>224</v>
       </c>
@@ -4730,15 +4721,15 @@
         <v>225</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B37" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
       <c r="A38" t="s">
         <v>132</v>
       </c>
@@ -4746,44 +4737,44 @@
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -4800,7 +4791,7 @@
     <hyperlink ref="E12" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
     <hyperlink ref="E13" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
     <hyperlink ref="E14" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
-    <hyperlink ref="D16" r:id="rId13" xr:uid="{A653A6B2-EC28-47BF-AD71-119E64575518}"/>
+    <hyperlink ref="D16" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -4815,28 +4806,28 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="28.85546875" customWidth="1"/>
-    <col min="2" max="2" width="41.5703125" customWidth="1"/>
-    <col min="3" max="3" width="100.85546875" customWidth="1"/>
-    <col min="4" max="4" width="73.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.8984375" customWidth="1"/>
+    <col min="2" max="2" width="41.59765625" customWidth="1"/>
+    <col min="3" max="3" width="100.8984375" customWidth="1"/>
+    <col min="4" max="4" width="73.69921875" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="57.5703125" customWidth="1"/>
+    <col min="6" max="6" width="38.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.69921875" customWidth="1"/>
+    <col min="8" max="8" width="19.59765625" customWidth="1"/>
+    <col min="9" max="9" width="57.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B1" s="6" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4865,24 +4856,24 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="16.8">
       <c r="A3" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B3" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>252</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F3" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -4891,15 +4882,15 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="16.8">
       <c r="A4" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B4" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>256</v>
@@ -4908,10 +4899,10 @@
         <v>257</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="F4" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -4920,537 +4911,537 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B6" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="C6" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="F6" t="s">
-        <v>299</v>
-      </c>
-      <c r="G6" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G6" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B7" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C7" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="F7" t="s">
-        <v>299</v>
-      </c>
-      <c r="G7" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G7" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B8" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C8" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="F8" t="s">
-        <v>299</v>
-      </c>
-      <c r="G8" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G8" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B9" t="s">
+        <v>313</v>
+      </c>
+      <c r="C9" t="s">
+        <v>314</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F9" t="s">
         <v>306</v>
       </c>
-      <c r="C9" t="s">
-        <v>307</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="F9" t="s">
-        <v>299</v>
-      </c>
-      <c r="G9" s="38" t="b">
+      <c r="G9" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B10" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C10" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="F10" t="s">
-        <v>299</v>
-      </c>
-      <c r="G10" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G10" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B11" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="C11" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="F11" t="s">
-        <v>299</v>
-      </c>
-      <c r="G11" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G11" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B12" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="C12" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="F12" t="s">
-        <v>299</v>
-      </c>
-      <c r="G12" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G12" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B13" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="C13" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="F13" t="s">
-        <v>299</v>
-      </c>
-      <c r="G13" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G13" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B14" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="C14" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="F14" t="s">
-        <v>299</v>
-      </c>
-      <c r="G14" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G14" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H14" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B15" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C15" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="F15" t="s">
-        <v>299</v>
-      </c>
-      <c r="G15" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G15" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H15" t="b">
         <v>0</v>
       </c>
       <c r="I15" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B18" s="43" t="s">
-        <v>326</v>
-      </c>
-      <c r="C18" s="43" t="s">
-        <v>327</v>
-      </c>
-      <c r="E18" s="44" t="s">
-        <v>328</v>
-      </c>
-      <c r="F18" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G18" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" s="43" t="b">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="3" customFormat="1">
+      <c r="A18" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G18" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B19" s="43" t="s">
-        <v>329</v>
-      </c>
-      <c r="C19" s="43" t="s">
-        <v>330</v>
-      </c>
-      <c r="E19" s="44" t="s">
-        <v>328</v>
-      </c>
-      <c r="F19" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G19" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="43" t="b">
+    <row r="19" spans="1:8" s="3" customFormat="1">
+      <c r="A19" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G19" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B20" s="43" t="s">
-        <v>331</v>
-      </c>
-      <c r="C20" s="43" t="s">
-        <v>332</v>
-      </c>
-      <c r="E20" s="44" t="s">
-        <v>333</v>
-      </c>
-      <c r="F20" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G20" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" s="43" t="b">
+    <row r="20" spans="1:8" s="3" customFormat="1">
+      <c r="A20" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G20" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B21" s="43" t="s">
-        <v>334</v>
-      </c>
-      <c r="C21" s="43" t="s">
-        <v>335</v>
-      </c>
-      <c r="E21" s="44" t="s">
-        <v>333</v>
-      </c>
-      <c r="F21" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G21" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" s="43" t="b">
+    <row r="21" spans="1:8" s="3" customFormat="1">
+      <c r="A21" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G21" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B22" s="43" t="s">
-        <v>336</v>
-      </c>
-      <c r="C22" s="43" t="s">
-        <v>337</v>
-      </c>
-      <c r="E22" s="44" t="s">
-        <v>338</v>
-      </c>
-      <c r="F22" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G22" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="43" t="b">
+    <row r="22" spans="1:8" s="3" customFormat="1">
+      <c r="A22" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G22" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="B23" s="43" t="s">
-        <v>339</v>
-      </c>
-      <c r="C23" s="43" t="s">
-        <v>340</v>
-      </c>
-      <c r="E23" s="44" t="s">
-        <v>341</v>
-      </c>
-      <c r="F23" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G23" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="43" t="b">
+    <row r="23" spans="1:8" s="3" customFormat="1">
+      <c r="A23" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G23" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>289</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>342</v>
+        <v>296</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>349</v>
       </c>
       <c r="C24" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="F24" t="s">
-        <v>299</v>
-      </c>
-      <c r="G24" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G24" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H24" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>289</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>345</v>
+        <v>296</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>352</v>
       </c>
       <c r="C25" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="F25" t="s">
-        <v>299</v>
-      </c>
-      <c r="G25" s="38" t="b">
+        <v>306</v>
+      </c>
+      <c r="G25" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H25" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>289</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="C26" s="39" t="s">
-        <v>349</v>
+        <v>296</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="C26" s="51" t="s">
+        <v>356</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="F26" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="B28" s="47" t="s">
-        <v>351</v>
-      </c>
-      <c r="C28" s="49" t="s">
-        <v>352</v>
-      </c>
-      <c r="D28" s="46"/>
-      <c r="E28" s="48" t="s">
-        <v>353</v>
-      </c>
-      <c r="F28" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G28" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H28" s="43" t="b">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="3" customFormat="1">
+      <c r="A28" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="B28" s="53" t="s">
+        <v>358</v>
+      </c>
+      <c r="C28" s="54" t="s">
+        <v>359</v>
+      </c>
+      <c r="D28" s="52"/>
+      <c r="E28" s="55" t="s">
+        <v>360</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G28" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="B29" s="47" t="s">
-        <v>354</v>
-      </c>
-      <c r="C29" s="49" t="s">
-        <v>355</v>
-      </c>
-      <c r="D29" s="43"/>
-      <c r="E29" s="44" t="s">
-        <v>356</v>
-      </c>
-      <c r="F29" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G29" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H29" s="43" t="b">
+    <row r="29" spans="1:8">
+      <c r="A29" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="B29" s="53" t="s">
+        <v>361</v>
+      </c>
+      <c r="C29" s="54" t="s">
+        <v>362</v>
+      </c>
+      <c r="D29" s="3"/>
+      <c r="E29" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G29" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="B30" s="47" t="s">
-        <v>357</v>
-      </c>
-      <c r="C30" s="49" t="s">
-        <v>358</v>
-      </c>
-      <c r="D30" s="43"/>
-      <c r="E30" s="44" t="s">
-        <v>359</v>
-      </c>
-      <c r="F30" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G30" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H30" s="43" t="b">
+    <row r="30" spans="1:8">
+      <c r="A30" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="B30" s="53" t="s">
+        <v>364</v>
+      </c>
+      <c r="C30" s="54" t="s">
+        <v>365</v>
+      </c>
+      <c r="D30" s="3"/>
+      <c r="E30" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G30" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="B31" s="50" t="s">
-        <v>334</v>
-      </c>
-      <c r="C31" s="49" t="s">
-        <v>360</v>
-      </c>
-      <c r="D31" s="43"/>
-      <c r="E31" s="44" t="s">
-        <v>361</v>
-      </c>
-      <c r="F31" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="G31" s="45" t="b">
-        <v>1</v>
-      </c>
-      <c r="H31" s="43" t="b">
+    <row r="31" spans="1:8">
+      <c r="A31" s="52" t="s">
+        <v>296</v>
+      </c>
+      <c r="B31" s="56" t="s">
+        <v>341</v>
+      </c>
+      <c r="C31" s="54" t="s">
+        <v>367</v>
+      </c>
+      <c r="D31" s="3"/>
+      <c r="E31" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G31" s="50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2">
       <c r="A33" t="s">
         <v>124</v>
       </c>
@@ -5458,12 +5449,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="40" t="s">
-        <v>362</v>
+    <row r="34" spans="1:2">
+      <c r="A34" s="57" t="s">
+        <v>369</v>
       </c>
       <c r="B34" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -5505,26 +5496,26 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3816B5CE-CC2D-4932-96C4-30D88CAD70AE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="50.69921875" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="82.140625" customWidth="1"/>
+    <col min="3" max="3" width="82.09765625" customWidth="1"/>
     <col min="4" max="4" width="110" customWidth="1"/>
-    <col min="5" max="9" width="50.7109375" customWidth="1"/>
+    <col min="5" max="9" width="50.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B1" s="6" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -5553,113 +5544,113 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>365</v>
-      </c>
-      <c r="B3" s="41" t="s">
-        <v>370</v>
+        <v>372</v>
+      </c>
+      <c r="B3" s="58" t="s">
+        <v>373</v>
       </c>
       <c r="C3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>372</v>
+      </c>
+      <c r="B4" s="58" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B5" s="58" t="s">
+        <v>377</v>
+      </c>
+      <c r="C5" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>365</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>369</v>
-      </c>
-      <c r="C4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>365</v>
-      </c>
-      <c r="B5" s="41" t="s">
-        <v>366</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>372</v>
+      </c>
+      <c r="B6" s="58" t="s">
         <v>379</v>
-      </c>
-      <c r="F5" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>365</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>367</v>
       </c>
       <c r="C6" t="s">
         <v>380</v>
       </c>
       <c r="F6" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>365</v>
-      </c>
-      <c r="B7" s="41" t="s">
-        <v>368</v>
+        <v>372</v>
+      </c>
+      <c r="B7" s="58" t="s">
+        <v>381</v>
       </c>
       <c r="C7" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F7" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>365</v>
-      </c>
-      <c r="B8" s="49" t="s">
-        <v>371</v>
+        <v>372</v>
+      </c>
+      <c r="B8" s="54" t="s">
+        <v>383</v>
       </c>
       <c r="C8" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="F8" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>365</v>
-      </c>
-      <c r="B9" s="49" t="s">
         <v>372</v>
       </c>
+      <c r="B9" s="54" t="s">
+        <v>385</v>
+      </c>
       <c r="C9" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="F9" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>365</v>
-      </c>
-      <c r="B10" s="49" t="s">
-        <v>373</v>
+        <v>372</v>
+      </c>
+      <c r="B10" s="54" t="s">
+        <v>387</v>
       </c>
       <c r="C10" t="s">
-        <v>375</v>
+        <v>388</v>
       </c>
       <c r="F10" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>124</v>
       </c>
@@ -5667,19 +5658,20 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="40" t="s">
-        <v>362</v>
+    <row r="18" spans="1:2">
+      <c r="A18" s="57" t="s">
+        <v>369</v>
       </c>
       <c r="B18" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1" r:id="rId1" xr:uid="{9E39D594-078A-45C7-AACA-459785887123}"/>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <tableParts count="2">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>

</xml_diff>

<commit_message>
excel update, ZOG, AUT
excel update, ZOG, AUT
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026_4sfera_com.xlsx
+++ b/AQD R3 DDBB views 2026_4sfera_com.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lallana\Desktop\Cambios R3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5220EFB-A9F4-4BAF-880C-D3574C18575A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1442F60B-5818-4D61-96E1-7B9AEE7D21CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6264" yWindow="720" windowWidth="17280" windowHeight="9024" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SamplingProcess (SPP)" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,9 @@
     <sheet name="SamplingPoint (SPO)" sheetId="3" r:id="rId3"/>
     <sheet name="SamplingPointLocation (SPL) " sheetId="4" r:id="rId4"/>
     <sheet name="ZoneGeometry (ZOG)" sheetId="5" r:id="rId5"/>
+    <sheet name="Authority (AUT)" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -38,65 +34,29 @@
   <commentList>
     <comment ref="B9" authorId="0" shapeId="0" xr:uid="{490B77A0-62D5-4524-8722-2821422E9730}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-I should replace this QA with two different QAs. 
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    I should replace this QA with two different QAs. 
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B21" authorId="1" shapeId="0" xr:uid="{98339C65-A981-4E71-B011-09FFEF030360}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Is this needed??? We have 07_A and we check if appears int he Vocabulary Table
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Is this needed??? We have 07_A and we check if appears int he Vocabulary Table
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B24" authorId="2" shapeId="0" xr:uid="{BC8092FB-ED06-4F30-BB5A-3740F72BE98B}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-I should replace this QA with two different QAs. 
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    I should replace this QA with two different QAs. 
 </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -113,65 +73,29 @@
   <commentList>
     <comment ref="B7" authorId="0" shapeId="0" xr:uid="{3DA4E063-7EDE-42C2-89DC-071A89E072CE}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-I think this QA is not correct. See “STA_07_A should be testing StationNationalCode (StationEoICode is tested in STA_02_ QC rules)” (see STA_02_B new)
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    I think this QA is not correct. See “STA_07_A should be testing StationNationalCode (StationEoICode is tested in STA_02_ QC rules)” (see STA_02_B new)
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B12" authorId="1" shapeId="0" xr:uid="{8FFECDF7-F7B5-415B-895C-2A49C7898D2E}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-I should replace this QA with two different QAs. 
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    I should replace this QA with two different QAs. 
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B14" authorId="2" shapeId="0" xr:uid="{30CCE20F-0910-4B3E-B84F-8FCC06678552}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-I think it’s necessary to create more QCs for this attribute
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    I think it’s necessary to create more QCs for this attribute
 </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -190,107 +114,47 @@
   <commentList>
     <comment ref="B3" authorId="0" shapeId="0" xr:uid="{3E8DD45C-46E7-465E-8876-4919E45020C6}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-It should be renamed as SPO_04_A because PollutantId is SPO_04
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It should be renamed as SPO_04_A because PollutantId is SPO_04
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B4" authorId="1" shapeId="0" xr:uid="{54D61B2D-210B-4D09-86A7-B45CE962A4B8}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-It should be renamed as SPO_04_B because PollutantId is SPO_04
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It should be renamed as SPO_04_B because PollutantId is SPO_04
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B5" authorId="2" shapeId="0" xr:uid="{E347F355-D485-4768-9BD7-1A96560682D0}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-It should be renamed as SPO_05_A because StationEoICode is SPO_05
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It should be renamed as SPO_05_A because StationEoICode is SPO_05
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B7" authorId="3" shapeId="0" xr:uid="{1E85BB37-0120-43BF-94F4-7A83479F1A4F}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-AirQualityStationArea has been moved to SPL
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    AirQualityStationArea has been moved to SPL
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B8" authorId="4" shapeId="0" xr:uid="{A573D4B5-DC98-495C-A577-BD4C21E95BCB}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-AirQualityStationArea has been moved to SPL
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    AirQualityStationArea has been moved to SPL
 </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -311,149 +175,65 @@
   <commentList>
     <comment ref="B18" authorId="0" shapeId="0" xr:uid="{20493F91-5BBC-482C-9C73-D643F028C2D4}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-We propose to merge both QA.
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    We propose to merge both QA.
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B20" authorId="1" shapeId="0" xr:uid="{52122516-33F3-4456-8E6E-9B680A5AD7E3}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-We propose to merge both QA.
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    We propose to merge both QA.
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B22" authorId="2" shapeId="0" xr:uid="{29CB7204-F2B2-4884-8A8B-64AE37F06BE6}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Now we have -10 and 5700
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Now we have -10 and 5700
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B23" authorId="3" shapeId="0" xr:uid="{BF0E0883-33BA-43E0-BF35-EC267681D38F}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-In the current QA we have 0-30 meters
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    In the current QA we have 0-30 meters
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B24" authorId="4" shapeId="0" xr:uid="{CF358EB7-C8E0-4BDE-AD85-1E5D278FC4A6}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B25" authorId="5" shapeId="0" xr:uid="{0A0E88C7-8798-478D-95CD-9D699DD4076D}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Mandatory SamplingPointCategory = Traffic
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Mandatory SamplingPointCategory = Traffic
 </t>
-        </r>
       </text>
     </comment>
     <comment ref="B26" authorId="6" shapeId="0" xr:uid="{680D8D74-A90F-40EB-8152-C2AC5B1BD190}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t>Comment:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
 </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -461,7 +241,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="426">
   <si>
     <t>2026 task</t>
   </si>
@@ -1727,16 +1507,539 @@
   <si>
     <t>Attribute ZOG_03 must use one of the supported coordinate reference systems: EPSG:3035, EPSG:4258 or EPSG:4326.</t>
   </si>
+  <si>
+    <t>ZoneGeometryGeoJson</t>
+  </si>
+  <si>
+    <t>ZOG_03</t>
+  </si>
+  <si>
+    <t>CREATED AS STA_09_A2 BECAUSE STA_09_A ALREADY EXISTED</t>
+  </si>
+  <si>
+    <t>CREATED AS STA_04_B2</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/306673</t>
+  </si>
+  <si>
+    <t>ZOG_03_D</t>
+  </si>
+  <si>
+    <t>The value reported under ZoneGeometry in the ZoneGeometry table shall be expressed using one of the supported coordinate reference systems.</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/306674</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <r>
+      <t>Task #306644</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_01_A Check country code</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306645</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_02_A AuthorityInstanceId</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306646</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_03_A - Doble check it looks into https://dd.eionet.europa.eu/vocabulary/aq/authorityrole</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306647</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_04_A email</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306648</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_05_A AuthorityInstance</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306649</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_06_A AuthorityName</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306650</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_07_A AuthorityURL - done in 2025</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306651</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_07_B AuthorityURL - done in 2025</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306652</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_08_A AuthorityAddress</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306653</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_09_A PersonName</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306654</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_10_A AuthorityStatus - done in 2025</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Task #306655</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: AUT_PK</t>
+    </r>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/306643</t>
+  </si>
+  <si>
+    <r>
+      <t>The value reported under </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>CountryCode</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t> in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>Authority</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t> table shall identify the reporting country or territory using a valid ISO2 country code.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/306644</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>R3 does this automatically</t>
+  </si>
+  <si>
+    <t>The same as 03_C?</t>
+  </si>
+  <si>
+    <t>need a reference table with the country codes and the coordinates.Function 'within'</t>
+  </si>
+  <si>
+    <t>https://taskman.eionet.europa.eu/issues/306645</t>
+  </si>
+  <si>
+    <t>The value reported under AuthorityInstanceId in the Authority table must satisfy conformity with the expected reference ID based on the associated AuthorityInstance type: If AuthorityInstance = 'nuts0' (id), then AuthorityInstanceId must match CountryCode in the same Authority table (AUT_01) [Notation]; If AuthorityInstance = 'nuts1-3' (id), then AuthorityInstanceId must match an existing ZoneId in the AssessmentRegimeZone table (ARZ_05) [Notation]; If AuthorityInstance = 'zone', then AuthorityInstanceId must match an existing ZoneId in the ZoneGeometry table (ZOG_02) [Notation]. See relationship between id and notation in</t>
+  </si>
+  <si>
+    <t>test AUT_02</t>
+  </si>
+  <si>
+    <t>USE [Airquality_R3]
+GO
+SET ANSI_NULLS ON
+GO
+SET QUOTED_IDENTIFIER ON
+GO
+CREATE VIEW [qc].[AUT_02_A] AS
+-- Creation date: 27 August 2025
+-- QC rule code: AUTH_02_A
+-- QC rule name: AUTH_02_A Cross-check - [AuthorityInstanceId] AUTH_01 ARZ_05 STA_03
+WITH CTE_authority AS (
+  SELECT 
+    LTRIM(RTRIM(NULLIF([authorityinstance], ''))) AS authorityinstance,
+    LTRIM(RTRIM(NULLIF([authorityinstanceid], ''))) AS authorityinstanceid,
+    LTRIM(RTRIM(NULLIF([countrycode], ''))) AS countrycode
+  FROM reporting.Authority
+  WHERE [authorityinstanceid] IS NOT NULL 
+    AND [authorityinstance] IS NOT NULL
+    AND [countrycode] IS NOT NULL
+),
+-- Data in reported tables?
+assessment_data_present AS (
+  SELECT CASE WHEN COUNT(*) &gt; 0 THEN 1 ELSE 0 END AS has_data 
+  FROM reporting.AssessmentRegimeZone
+),
+station_data_present AS (
+  SELECT CASE WHEN COUNT(*) &gt; 0 THEN 1 ELSE 0 END AS has_data 
+  FROM reporting.MeasurementStation
+),
+-- Valid zones (reference if table is not reported)
+CTE_zones AS (
+  SELECT DISTINCT LTRIM(RTRIM([zoneid])) AS zoneid
+  FROM (
+    SELECT [zoneid] FROM reporting.AssessmentRegimeZone
+    WHERE (SELECT has_data FROM assessment_data_present) = 1
+    UNION ALL
+    SELECT [zoneid] FROM reference.AssessmentRegimeZone
+    WHERE (SELECT has_data FROM assessment_data_present) = 0
+  ) t
+),
+-- Valid network (reference if table is not reported)
+CTE_networks AS (
+  SELECT DISTINCT LTRIM(RTRIM([NetworkId])) AS airqualitynetwork
+  FROM (
+    SELECT [NetworkId] FROM reporting.MeasurementStation
+    WHERE (SELECT has_data FROM station_data_present) = 1
+    UNION ALL
+    SELECT [NetworkId] FROM reference.MeasurementStation
+    WHERE (SELECT has_data FROM station_data_present) = 0
+  ) t
+),
+-- AUTH_01: If instance = 'nuts0',  countrycode
+CTE_invalid_nuts0 AS (
+  SELECT *
+  FROM CTE_authority
+  WHERE authorityinstance = 'nuts0'
+    AND authorityinstanceid &lt;&gt; countrycode
+),
+-- ARZ_05: zone/nuts(1-3) , zoneid
+CTE_invalid_zones AS (
+  SELECT *
+  FROM CTE_authority a
+  WHERE (authorityinstance = 'zone' 
+       OR authorityinstance LIKE 'nuts1' 
+       OR authorityinstance LIKE 'nuts2' 
+       OR authorityinstance LIKE 'nuts3')
+    AND NOT EXISTS (
+      SELECT 1 FROM CTE_zones z
+      WHERE z.zoneid = a.authorityinstanceid
+    )
+),
+-- STA_03: network, airqualitynetwork
+CTE_invalid_networks AS (
+  SELECT *
+  FROM CTE_authority a
+  WHERE authorityinstance = 'network'
+    AND NOT EXISTS (
+      SELECT 1 FROM CTE_networks s
+      WHERE s.airqualitynetwork = a.authorityinstanceid
+    )
+)
+-- RESULT
+SELECT 'AUTH_01' AS rule_violation, * FROM CTE_invalid_nuts0
+UNION ALL
+SELECT 'ARZ_05' AS rule_violation, * FROM CTE_invalid_zones
+UNION ALL
+SELECT 'STA_03' AS rule_violation, * FROM CTE_invalid_networks
+;
+GO</t>
+  </si>
+  <si>
+    <r>
+      <t>AuthorityRole</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF333333"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>field does not exist in authority table</t>
+    </r>
+  </si>
+  <si>
+    <t>USE [Airquality_R3];
+GO
+SET ANSI_NULLS ON;
+GO
+SET QUOTED_IDENTIFIER ON;
+GO
+CREATE OR ALTER VIEW [qc].[AUTH_03_A]
+AS
+-- QC rule code: AUTH_03_A
+-- QC rule name: Vocabulary - [AuthorityRole]
+WITH CTE_authority AS
+(
+    SELECT
+        NULLIF(LTRIM(RTRIM([authorityrole])), '') AS authorityrole
+    FROM reporting.Authority
+),
+missing_codes AS
+(
+    SELECT
+        a.authorityrole
+    FROM CTE_authority AS a
+    LEFT JOIN reference.Vocabulary AS v
+        ON a.authorityrole COLLATE Latin1_General_CI_AS
+         = v.[notation] COLLATE Latin1_General_CI_AS
+       AND v.[vocabulary] = 'authorityrole'
+    WHERE a.authorityrole IS NOT NULL
+      AND v.[notation] IS NULL
+)
+SELECT
+    authorityrole
+FROM missing_codes;
+GO</t>
+  </si>
+  <si>
+    <t>test AUT_03 (field not exist)</t>
+  </si>
+  <si>
+    <t>USE [Airquality_R3];
+GO
+SET ANSI_NULLS ON;
+GO
+SET QUOTED_IDENTIFIER ON;
+GO
+CREATE OR ALTER VIEW [qc].[AUT_04_A]
+AS
+-- QC rule code: AUT_04_A
+-- QC rule name: Format validation - [Email]
+WITH CTE_authority AS
+(
+    SELECT
+        NULLIF([Email], '') AS Email
+    FROM reporting.Authority
+),
+CTE_email_parts AS
+(
+    SELECT
+        a.Email,
+        CHARINDEX('@', a.Email) AS at_position,
+        LEN(a.Email) - LEN(REPLACE(a.Email, '@', '')) AS at_count
+    FROM CTE_authority AS a
+    WHERE a.Email IS NOT NULL
+),
+CTE_invalid_emails AS
+(
+    SELECT
+        e.Email
+    FROM CTE_email_parts AS e
+    CROSS APPLY
+    (
+        SELECT
+            LEFT(e.Email, e.at_position - 1) AS local_part,
+            SUBSTRING(e.Email, e.at_position + 1, LEN(e.Email)) AS domain_part
+    ) AS p
+    WHERE
+        -- The email address must contain exactly one @ symbol.
+        e.at_count &lt;&gt; 1
+        -- Both the local part and domain part must contain a value.
+        OR e.at_position &lt;= 1
+        OR e.at_position &gt;= LEN(e.Email)
+        -- Spaces are not allowed.
+        OR CHARINDEX(' ', e.Email) &gt; 0
+        -- Allowed local-part characters: letters, digits, dot, underscore,
+        -- percent sign, plus sign and hyphen.
+        OR p.local_part COLLATE Latin1_General_100_BIN2
+           LIKE '%[^A-Za-z0-9._%+-]%'
+        -- The local part cannot start or end with a dot,
+        -- and cannot contain consecutive dots.
+        OR p.local_part LIKE '.%'
+        OR p.local_part LIKE '%.'
+        OR p.local_part LIKE '%..%'
+        -- The domain part must include at least one dot.
+        OR CHARINDEX('.', p.domain_part) = 0
+        -- Allowed domain characters: letters, digits, dot and hyphen.
+        OR p.domain_part COLLATE Latin1_General_100_BIN2
+           LIKE '%[^A-Za-z0-9.-]%'
+        -- The domain cannot start or end with a dot or hyphen,
+        -- and cannot contain consecutive dots.
+        OR p.domain_part LIKE '.%'
+        OR p.domain_part LIKE '%.'
+        OR p.domain_part LIKE '-%'
+        OR p.domain_part LIKE '%-'
+        OR p.domain_part LIKE '%..%'
+)
+SELECT
+    Email
+FROM CTE_invalid_emails;
+GO</t>
+  </si>
+  <si>
+    <t>test AUT_04</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1822,15 +2125,49 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <name val="Tahoma"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Verdana"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1939,8 +2276,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -2011,93 +2360,114 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2105,7 +2475,53 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFDD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2234,24 +2650,24 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="tc={98339c65-a981-4e71-b011-09ffef030360}" id="{2FFCC802-290F-A181-67E9-9C1FB06B16B7}"/>
-  <person displayName="tc={bc8092fb-ed06-4f30-bb5a-3740f72be98b}" id="{3B10C98B-12F6-CEA5-663B-22D5674EBE2A}"/>
-  <person displayName="tc={490b77a0-62d5-4524-8722-2821422e9730}" id="{1B31B7B1-7F12-2A29-CFB1-49CF8E7C8D1B}"/>
-  <person displayName="tc={8ffecdf7-f7b5-415b-895c-2a49c7898d2e}" id="{4BA197E0-565D-B4CD-48F6-892443E0FE5A}"/>
-  <person displayName="tc={30cce20f-0910-4b3e-b84f-8fcc06678552}" id="{4533ACC3-D2D9-421D-E2D9-DD5BBC954281}"/>
-  <person displayName="tc={3da4e063-7ede-42c2-89dc-071a89e072ce}" id="{B86E3BCE-DB44-F70C-4F19-A905D2C6DA35}"/>
-  <person displayName="tc={3e8dd45c-46e7-465e-8876-4919e45020c6}" id="{C5B26D5A-1FAB-CCEB-1798-409D1CA99359}"/>
-  <person displayName="tc={54d61b2d-210b-4d09-86a7-b45ce962a4b8}" id="{B357EAE8-074C-556E-B445-E557AC811191}"/>
-  <person displayName="tc={e347f355-d485-4768-9bd7-1a96560682d0}" id="{A2E2009C-EA6B-4971-F6E3-5A907E3C75EF}"/>
-  <person displayName="tc={1e85bb37-0120-43bf-94f4-7a83479f1a4f}" id="{90F399EE-5AD3-4BB5-4CB3-5AC18E1730C2}"/>
-  <person displayName="tc={a573d4b5-dc98-495c-a577-bd4c21e95bcb}" id="{213A65BA-8F48-8AFF-71F5-22CCA5765ACD}"/>
-  <person displayName="tc={20493f91-5bbc-482c-9c73-d643f028c2d4}" id="{9E5FF495-DF5E-8E27-8D51-71042DA4EE85}"/>
-  <person displayName="tc={52122516-33f3-4456-8e6e-9b680a5ad7e3}" id="{2C5FE0D2-EA13-B987-FA4A-10E40558B40F}"/>
-  <person displayName="tc={29cb7204-f2b2-4884-8a8b-64ae37f06be6}" id="{83940ACE-E867-47D2-FC2B-B9DC6DDE3EB5}"/>
-  <person displayName="tc={bf0e0883-33ba-43e0-bf35-ec267681d38f}" id="{C98B2C38-5018-19BA-51C9-F28AAF6A12C7}"/>
-  <person displayName="tc={cf358eb7-c8e0-4bde-ad85-1e5d278fc4a6}" id="{4566558B-34AE-FCD8-B670-0A7AB2298808}"/>
-  <person displayName="tc={0a0e88c7-8798-478d-95cd-9d699dd4076d}" id="{34F2EA13-14CC-C373-F261-EBD239A18C63}"/>
-  <person displayName="tc={680d8d74-a90f-40eb-8152-c2ac5b1bd190}" id="{1E054922-84FC-8C7E-BDBC-C675B6FCA1B2}"/>
+  <person displayName="tc={0a0e88c7-8798-478d-95cd-9d699dd4076d}" id="{34F2EA13-14CC-C373-F261-EBD239A18C63}" userId="" providerId=""/>
+  <person displayName="tc={1e85bb37-0120-43bf-94f4-7a83479f1a4f}" id="{90F399EE-5AD3-4BB5-4CB3-5AC18E1730C2}" userId="" providerId=""/>
+  <person displayName="tc={20493f91-5bbc-482c-9c73-d643f028c2d4}" id="{9E5FF495-DF5E-8E27-8D51-71042DA4EE85}" userId="" providerId=""/>
+  <person displayName="tc={29cb7204-f2b2-4884-8a8b-64ae37f06be6}" id="{83940ACE-E867-47D2-FC2B-B9DC6DDE3EB5}" userId="" providerId=""/>
+  <person displayName="tc={30cce20f-0910-4b3e-b84f-8fcc06678552}" id="{4533ACC3-D2D9-421D-E2D9-DD5BBC954281}" userId="" providerId=""/>
+  <person displayName="tc={3da4e063-7ede-42c2-89dc-071a89e072ce}" id="{B86E3BCE-DB44-F70C-4F19-A905D2C6DA35}" userId="" providerId=""/>
+  <person displayName="tc={3e8dd45c-46e7-465e-8876-4919e45020c6}" id="{C5B26D5A-1FAB-CCEB-1798-409D1CA99359}" userId="" providerId=""/>
+  <person displayName="tc={490b77a0-62d5-4524-8722-2821422e9730}" id="{1B31B7B1-7F12-2A29-CFB1-49CF8E7C8D1B}" userId="" providerId=""/>
+  <person displayName="tc={52122516-33f3-4456-8e6e-9b680a5ad7e3}" id="{2C5FE0D2-EA13-B987-FA4A-10E40558B40F}" userId="" providerId=""/>
+  <person displayName="tc={54d61b2d-210b-4d09-86a7-b45ce962a4b8}" id="{B357EAE8-074C-556E-B445-E557AC811191}" userId="" providerId=""/>
+  <person displayName="tc={680d8d74-a90f-40eb-8152-c2ac5b1bd190}" id="{1E054922-84FC-8C7E-BDBC-C675B6FCA1B2}" userId="" providerId=""/>
+  <person displayName="tc={8ffecdf7-f7b5-415b-895c-2a49c7898d2e}" id="{4BA197E0-565D-B4CD-48F6-892443E0FE5A}" userId="" providerId=""/>
+  <person displayName="tc={98339c65-a981-4e71-b011-09ffef030360}" id="{2FFCC802-290F-A181-67E9-9C1FB06B16B7}" userId="" providerId=""/>
+  <person displayName="tc={a573d4b5-dc98-495c-a577-bd4c21e95bcb}" id="{213A65BA-8F48-8AFF-71F5-22CCA5765ACD}" userId="" providerId=""/>
+  <person displayName="tc={bc8092fb-ed06-4f30-bb5a-3740f72be98b}" id="{3B10C98B-12F6-CEA5-663B-22D5674EBE2A}" userId="" providerId=""/>
+  <person displayName="tc={bf0e0883-33ba-43e0-bf35-ec267681d38f}" id="{C98B2C38-5018-19BA-51C9-F28AAF6A12C7}" userId="" providerId=""/>
+  <person displayName="tc={cf358eb7-c8e0-4bde-ad85-1e5d278fc4a6}" id="{4566558B-34AE-FCD8-B670-0A7AB2298808}" userId="" providerId=""/>
+  <person displayName="tc={e347f355-d485-4768-9bd7-1a96560682d0}" id="{A2E2009C-EA6B-4971-F6E3-5A907E3C75EF}" userId="" providerId=""/>
 </personList>
 </file>
 
@@ -2284,6 +2700,22 @@
 </table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0BC4E8C3-85C6-489D-BF2D-740644FE565C}" name="Table11" displayName="Table11" ref="A2:G14" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3">
+  <autoFilter ref="A2:G14" xr:uid="{0BC4E8C3-85C6-489D-BF2D-740644FE565C}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{FCB4B3CE-80E1-443E-8E4E-D4DAF8DBF592}" name="QC rule" dataDxfId="1" dataCellStyle="Hyperlink"/>
+    <tableColumn id="2" xr3:uid="{F270D045-3F54-41FB-B521-15F84117A486}" name="Description"/>
+    <tableColumn id="3" xr3:uid="{9F2AADD6-BEE8-40A8-983C-2459092F782C}" name="Task"/>
+    <tableColumn id="4" xr3:uid="{A35617F8-F712-4679-B5D7-2B7086D1C24B}" name="Task 2"/>
+    <tableColumn id="5" xr3:uid="{C44348C3-0F88-457D-BED7-E1BA45C7CBEE}" name="Status"/>
+    <tableColumn id="6" xr3:uid="{100A1DEE-73E4-482C-A57F-2E84BD0A062E}" name="Github"/>
+    <tableColumn id="7" xr3:uid="{D0B66E62-673E-41AA-A120-FB808FA58CB9}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table469" displayName="Table469" ref="A35:B45">
   <autoFilter ref="A35:B45" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
@@ -2299,15 +2731,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table13" displayName="Table13" ref="A2:I22">
   <autoFilter ref="A2:I22" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Table" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="QC rule" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Description" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Task" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Task2" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Status" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Github" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Tested" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="Comments" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Table" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="QC rule" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Description" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Task" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Task2" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Status" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Github" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Tested" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="Comments" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2317,8 +2749,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table46" displayName="Table46" ref="A24:B28">
   <autoFilter ref="A24:B28" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="OLD name" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="NEW name" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="OLD name" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="NEW name" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2361,7 +2793,7 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="QC rule"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Description"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Task"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Task 2" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Task 2" dataDxfId="4"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Status"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="Github"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="Tested"/>
@@ -2383,8 +2815,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Table134710" displayName="Table134710" ref="A2:I10">
-  <autoFilter ref="A2:I10" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Table134710" displayName="Table134710" ref="A2:I11">
+  <autoFilter ref="A2:I11" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Table"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="QC rule"/>
@@ -2618,15 +3050,15 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B21" dT="2026-07-08T07:18:15.56Z" personId="{2ffcc802-290f-a181-67e9-9c1fb06b16b7}" id="{98339c65-a981-4e71-b011-09ffef030360}" done="0">
+  <threadedComment ref="B9" dT="2026-07-08T08:39:09.89" personId="{1B31B7B1-7F12-2A29-CFB1-49CF8E7C8D1B}" id="{490B77A0-62D5-4524-8722-2821422E9730}">
+    <text xml:space="preserve">I should replace this QA with two different QAs. 
+</text>
+  </threadedComment>
+  <threadedComment ref="B21" dT="2026-07-08T07:18:15.56" personId="{2FFCC802-290F-A181-67E9-9C1FB06B16B7}" id="{98339C65-A981-4E71-B011-09FFEF030360}">
     <text xml:space="preserve">Is this needed??? We have 07_A and we check if appears int he Vocabulary Table
 </text>
   </threadedComment>
-  <threadedComment ref="B24" dT="2026-07-08T08:38:26.82Z" personId="{3b10c98b-12f6-cea5-663b-22d5674ebe2a}" id="{bc8092fb-ed06-4f30-bb5a-3740f72be98b}" done="0">
-    <text xml:space="preserve">I should replace this QA with two different QAs. 
-</text>
-  </threadedComment>
-  <threadedComment ref="B9" dT="2026-07-08T08:39:09.89Z" personId="{1b31b7b1-7f12-2a29-cfb1-49cf8e7c8d1b}" id="{490b77a0-62d5-4524-8722-2821422e9730}" done="0">
+  <threadedComment ref="B24" dT="2026-07-08T08:38:26.82" personId="{3B10C98B-12F6-CEA5-663B-22D5674EBE2A}" id="{BC8092FB-ED06-4F30-BB5A-3740F72BE98B}">
     <text xml:space="preserve">I should replace this QA with two different QAs. 
 </text>
   </threadedComment>
@@ -2635,16 +3067,16 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B12" dT="2026-07-07T11:47:46.10Z" personId="{4ba197e0-565d-b4cd-48f6-892443e0fe5a}" id="{8ffecdf7-f7b5-415b-895c-2a49c7898d2e}" done="0">
+  <threadedComment ref="B7" dT="2026-07-07T11:37:08.34" personId="{B86E3BCE-DB44-F70C-4F19-A905D2C6DA35}" id="{3DA4E063-7EDE-42C2-89DC-071A89E072CE}">
+    <text xml:space="preserve">I think this QA is not correct. See “STA_07_A should be testing StationNationalCode (StationEoICode is tested in STA_02_ QC rules)” (see STA_02_B new)
+</text>
+  </threadedComment>
+  <threadedComment ref="B12" dT="2026-07-07T11:47:46.10" personId="{4BA197E0-565D-B4CD-48F6-892443E0FE5A}" id="{8FFECDF7-F7B5-415B-895C-2A49C7898D2E}">
     <text xml:space="preserve">I should replace this QA with two different QAs. 
 </text>
   </threadedComment>
-  <threadedComment ref="B14" dT="2026-07-07T11:53:25.68Z" personId="{4533acc3-d2d9-421d-e2d9-dd5bbc954281}" id="{30cce20f-0910-4b3e-b84f-8fcc06678552}" done="0">
+  <threadedComment ref="B14" dT="2026-07-07T11:53:25.68" personId="{4533ACC3-D2D9-421D-E2D9-DD5BBC954281}" id="{30CCE20F-0910-4B3E-B84F-8FCC06678552}">
     <text xml:space="preserve">I think it’s necessary to create more QCs for this attribute
-</text>
-  </threadedComment>
-  <threadedComment ref="B7" dT="2026-07-07T11:37:08.34Z" personId="{b86e3bce-db44-f70c-4f19-a905d2c6da35}" id="{3da4e063-7ede-42c2-89dc-071a89e072ce}" done="0">
-    <text xml:space="preserve">I think this QA is not correct. See “STA_07_A should be testing StationNationalCode (StationEoICode is tested in STA_02_ QC rules)” (see STA_02_B new)
 </text>
   </threadedComment>
 </ThreadedComments>
@@ -2652,23 +3084,23 @@
 
 <file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B3" dT="2026-07-07T12:24:03.07Z" personId="{c5b26d5a-1fab-cceb-1798-409d1ca99359}" id="{3e8dd45c-46e7-465e-8876-4919e45020c6}" done="0">
+  <threadedComment ref="B3" dT="2026-07-07T12:24:03.07" personId="{C5B26D5A-1FAB-CCEB-1798-409D1CA99359}" id="{3E8DD45C-46E7-465E-8876-4919E45020C6}">
     <text xml:space="preserve">It should be renamed as SPO_04_A because PollutantId is SPO_04
 </text>
   </threadedComment>
-  <threadedComment ref="B4" dT="2026-07-07T12:34:08.20Z" personId="{b357eae8-074c-556e-b445-e557ac811191}" id="{54d61b2d-210b-4d09-86a7-b45ce962a4b8}" done="0">
+  <threadedComment ref="B4" dT="2026-07-07T12:34:08.20" personId="{B357EAE8-074C-556E-B445-E557AC811191}" id="{54D61B2D-210B-4D09-86A7-B45CE962A4B8}">
     <text xml:space="preserve">It should be renamed as SPO_04_B because PollutantId is SPO_04
 </text>
   </threadedComment>
-  <threadedComment ref="B5" dT="2026-07-08T06:08:12.99Z" personId="{a2e2009c-ea6b-4971-f6e3-5a907e3c75ef}" id="{e347f355-d485-4768-9bd7-1a96560682d0}" done="0">
+  <threadedComment ref="B5" dT="2026-07-08T06:08:12.99" personId="{A2E2009C-EA6B-4971-F6E3-5A907E3C75EF}" id="{E347F355-D485-4768-9BD7-1A96560682D0}">
     <text xml:space="preserve">It should be renamed as SPO_05_A because StationEoICode is SPO_05
 </text>
   </threadedComment>
-  <threadedComment ref="B7" dT="2026-07-07T12:20:54.40Z" personId="{90f399ee-5ad3-4bb5-4cb3-5ac18e1730c2}" id="{1e85bb37-0120-43bf-94f4-7a83479f1a4f}" done="0">
+  <threadedComment ref="B7" dT="2026-07-07T12:20:54.40" personId="{90F399EE-5AD3-4BB5-4CB3-5AC18E1730C2}" id="{1E85BB37-0120-43BF-94F4-7A83479F1A4F}">
     <text xml:space="preserve">AirQualityStationArea has been moved to SPL
 </text>
   </threadedComment>
-  <threadedComment ref="B8" dT="2026-07-07T12:20:59.37Z" personId="{213a65ba-8f48-8aff-71f5-22cca5765acd}" id="{a573d4b5-dc98-495c-a577-bd4c21e95bcb}" done="0">
+  <threadedComment ref="B8" dT="2026-07-07T12:20:59.37" personId="{213A65BA-8F48-8AFF-71F5-22CCA5765ACD}" id="{A573D4B5-DC98-495C-A577-BD4C21E95BCB}">
     <text xml:space="preserve">AirQualityStationArea has been moved to SPL
 </text>
   </threadedComment>
@@ -2677,31 +3109,31 @@
 
 <file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B18" dT="2026-07-08T06:27:09.26Z" personId="{9e5ff495-df5e-8e27-8d51-71042da4ee85}" id="{20493f91-5bbc-482c-9c73-d643f028c2d4}" done="0">
+  <threadedComment ref="B18" dT="2026-07-08T06:27:09.26" personId="{9E5FF495-DF5E-8E27-8D51-71042DA4EE85}" id="{20493F91-5BBC-482C-9C73-D643F028C2D4}">
     <text xml:space="preserve">We propose to merge both QA.
 </text>
   </threadedComment>
-  <threadedComment ref="B20" dT="2026-07-08T06:27:18.69Z" personId="{2c5fe0d2-ea13-b987-fa4a-10e40558b40f}" id="{52122516-33f3-4456-8e6e-9b680a5ad7e3}" done="0">
+  <threadedComment ref="B20" dT="2026-07-08T06:27:18.69" personId="{2C5FE0D2-EA13-B987-FA4A-10E40558B40F}" id="{52122516-33F3-4456-8E6E-9B680A5AD7E3}">
     <text xml:space="preserve">We propose to merge both QA.
 </text>
   </threadedComment>
-  <threadedComment ref="B22" dT="2026-07-08T06:30:12.04Z" personId="{83940ace-e867-47d2-fc2b-b9dc6dde3eb5}" id="{29cb7204-f2b2-4884-8a8b-64ae37f06be6}" done="0">
+  <threadedComment ref="B22" dT="2026-07-08T06:30:12.04" personId="{83940ACE-E867-47D2-FC2B-B9DC6DDE3EB5}" id="{29CB7204-F2B2-4884-8A8B-64AE37F06BE6}">
     <text xml:space="preserve">Now we have -10 and 5700
 </text>
   </threadedComment>
-  <threadedComment ref="B23" dT="2026-07-08T06:31:17.86Z" personId="{c98b2c38-5018-19ba-51c9-f28aaf6a12c7}" id="{bf0e0883-33ba-43e0-bf35-ec267681d38f}" done="0">
+  <threadedComment ref="B23" dT="2026-07-08T06:31:17.86" personId="{C98B2C38-5018-19BA-51C9-F28AAF6A12C7}" id="{BF0E0883-33BA-43E0-BF35-EC267681D38F}">
     <text xml:space="preserve">In the current QA we have 0-30 meters
 </text>
   </threadedComment>
-  <threadedComment ref="B24" dT="2026-07-08T06:43:57.31Z" personId="{4566558b-34ae-fcd8-b670-0a7ab2298808}" id="{cf358eb7-c8e0-4bde-ad85-1e5d278fc4a6}" done="0">
+  <threadedComment ref="B24" dT="2026-07-08T06:43:57.31" personId="{4566558B-34AE-FCD8-B670-0A7AB2298808}" id="{CF358EB7-C8E0-4BDE-AD85-1E5D278FC4A6}">
     <text xml:space="preserve">It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
 </text>
   </threadedComment>
-  <threadedComment ref="B25" dT="2026-07-08T06:44:12.64Z" personId="{34f2ea13-14cc-c373-f261-ebd239a18c63}" id="{0a0e88c7-8798-478d-95cd-9d699dd4076d}" done="0">
+  <threadedComment ref="B25" dT="2026-07-08T06:44:12.64" personId="{34F2EA13-14CC-C373-F261-EBD239A18C63}" id="{0A0E88C7-8798-478D-95CD-9D699DD4076D}">
     <text xml:space="preserve">Mandatory SamplingPointCategory = Traffic
 </text>
   </threadedComment>
-  <threadedComment ref="B26" dT="2026-07-08T06:44:58.31Z" personId="{1e054922-84fc-8c7e-bdbc-c675b6fca1b2}" id="{680d8d74-a90f-40eb-8152-c2ac5b1bd190}" done="0">
+  <threadedComment ref="B26" dT="2026-07-08T06:44:58.31" personId="{1E054922-84FC-8C7E-BDBC-C675B6FCA1B2}" id="{680D8D74-A90F-40EB-8152-C2AC5B1BD190}">
     <text xml:space="preserve">It needs to be decided whether reporting it should be mandatory for all SamplingPointCategory values. 
 </text>
   </threadedComment>
@@ -2711,16 +3143,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I51"/>
-  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.09765625" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="104" customWidth="1"/>
-    <col min="4" max="4" width="52.8984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.8984375" customWidth="1"/>
+    <col min="3" max="3" width="61.140625" customWidth="1"/>
+    <col min="4" max="4" width="42.28515625" customWidth="1"/>
+    <col min="5" max="5" width="52.85546875" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="8" width="13.3984375" customWidth="1"/>
-    <col min="9" max="9" width="71.69921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.42578125" customWidth="1"/>
+    <col min="9" max="9" width="71.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -2760,7 +3192,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.8">
+    <row r="3" spans="1:9" ht="16.5">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3321,128 +3753,128 @@
       <c r="A25" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="11" t="s">
+      <c r="D25" s="9"/>
+      <c r="E25" s="10" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.6">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:9" ht="15.75">
+      <c r="A26" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="11" t="s">
+      <c r="D26" s="9"/>
+      <c r="E26" s="10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="10"/>
-      <c r="E27" s="11" t="s">
+      <c r="D27" s="9"/>
+      <c r="E27" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="59" customFormat="1">
-      <c r="A28" s="59" t="s">
+    <row r="28" spans="1:9" s="58" customFormat="1">
+      <c r="A28" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="59" t="s">
+      <c r="B28" s="58" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="59" t="s">
+      <c r="C28" s="58" t="s">
         <v>109</v>
       </c>
-      <c r="E28" s="60" t="s">
+      <c r="E28" s="59" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="59" customFormat="1">
-      <c r="A29" s="59" t="s">
+    <row r="29" spans="1:9" s="58" customFormat="1">
+      <c r="A29" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="59" t="s">
+      <c r="B29" s="58" t="s">
         <v>111</v>
       </c>
-      <c r="C29" s="59" t="s">
+      <c r="C29" s="58" t="s">
         <v>112</v>
       </c>
-      <c r="E29" s="60" t="s">
+      <c r="E29" s="59" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="59" customFormat="1">
-      <c r="A30" s="59" t="s">
+    <row r="30" spans="1:9" s="58" customFormat="1">
+      <c r="A30" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B30" s="59" t="s">
+      <c r="B30" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="C30" s="59" t="s">
+      <c r="C30" s="58" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="60" t="s">
+      <c r="E30" s="59" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="59" customFormat="1">
-      <c r="A31" s="59" t="s">
+    <row r="31" spans="1:9" s="58" customFormat="1">
+      <c r="A31" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B31" s="59" t="s">
+      <c r="B31" s="58" t="s">
         <v>116</v>
       </c>
-      <c r="C31" s="59" t="s">
+      <c r="C31" s="58" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="60" t="s">
+      <c r="E31" s="59" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="59" customFormat="1">
-      <c r="A32" s="59" t="s">
+    <row r="32" spans="1:9" s="58" customFormat="1">
+      <c r="A32" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="59" t="s">
+      <c r="B32" s="58" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="59" t="s">
+      <c r="C32" s="58" t="s">
         <v>119</v>
       </c>
-      <c r="E32" s="60" t="s">
+      <c r="E32" s="59" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="59" customFormat="1">
-      <c r="A33" s="59" t="s">
+    <row r="33" spans="1:5" s="58" customFormat="1">
+      <c r="A33" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="59" t="s">
+      <c r="B33" s="58" t="s">
         <v>121</v>
       </c>
-      <c r="C33" s="59" t="s">
+      <c r="C33" s="58" t="s">
         <v>122</v>
       </c>
-      <c r="E33" s="60" t="s">
+      <c r="E33" s="59" t="s">
         <v>123</v>
       </c>
     </row>
@@ -3503,8 +3935,8 @@
       <c r="A42" t="s">
         <v>135</v>
       </c>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="12"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
@@ -3528,10 +3960,10 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="14"/>
+      <c r="A46" s="13"/>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="15" t="s">
+      <c r="A48" s="14" t="s">
         <v>63</v>
       </c>
       <c r="B48" t="s">
@@ -3539,10 +3971,10 @@
       </c>
     </row>
     <row r="49" spans="1:3">
-      <c r="A49" s="16" t="s">
+      <c r="A49" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="16" t="s">
         <v>94</v>
       </c>
       <c r="C49" t="s">
@@ -3550,10 +3982,10 @@
       </c>
     </row>
     <row r="50" spans="1:3">
-      <c r="A50" s="15" t="s">
+      <c r="A50" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B50" s="15" t="s">
         <v>142</v>
       </c>
       <c r="C50" t="s">
@@ -3561,10 +3993,10 @@
       </c>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51" s="16" t="s">
+      <c r="A51" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="B51" s="16" t="s">
+      <c r="B51" s="15" t="s">
         <v>142</v>
       </c>
       <c r="C51" t="s">
@@ -3611,16 +4043,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="34.296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.09765625" customWidth="1"/>
-    <col min="3" max="3" width="102.3984375" customWidth="1"/>
-    <col min="4" max="4" width="52.8984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.8984375" customWidth="1"/>
-    <col min="6" max="6" width="47.09765625" customWidth="1"/>
-    <col min="7" max="8" width="13.3984375" customWidth="1"/>
-    <col min="9" max="9" width="185.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="3" max="3" width="102.42578125" customWidth="1"/>
+    <col min="4" max="4" width="52.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.85546875" customWidth="1"/>
+    <col min="6" max="6" width="47.140625" customWidth="1"/>
+    <col min="7" max="8" width="13.42578125" customWidth="1"/>
+    <col min="9" max="9" width="185.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -3667,13 +4099,13 @@
       <c r="B3" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>147</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>149</v>
       </c>
       <c r="F3" t="s">
@@ -3685,7 +4117,7 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="19" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3696,13 +4128,13 @@
       <c r="B4" t="s">
         <v>152</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>153</v>
       </c>
       <c r="D4" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>155</v>
       </c>
       <c r="F4" t="s">
@@ -3719,10 +4151,10 @@
       <c r="A5" t="s">
         <v>145</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="20" t="s">
         <v>158</v>
       </c>
       <c r="D5" s="6" t="s">
@@ -3741,53 +4173,53 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="23" customFormat="1">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:9" s="22" customFormat="1">
+      <c r="A6" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="G6" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" s="25" customFormat="1">
-      <c r="A7" s="25" t="s">
+      <c r="G6" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="24" customFormat="1">
+      <c r="A7" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="E7" s="26"/>
-      <c r="F7" s="25" t="s">
+      <c r="E7" s="25"/>
+      <c r="F7" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="G7" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="25" t="s">
+      <c r="G7" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="24" t="s">
         <v>170</v>
       </c>
     </row>
@@ -3798,13 +4230,13 @@
       <c r="B8" t="s">
         <v>171</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>13</v>
       </c>
       <c r="D8" t="s">
         <v>172</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="21" t="s">
         <v>173</v>
       </c>
       <c r="F8" t="s">
@@ -3824,7 +4256,7 @@
       <c r="B9" t="s">
         <v>175</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="20" t="s">
         <v>176</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -3850,7 +4282,7 @@
       <c r="B10" t="s">
         <v>179</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="20" t="s">
         <v>180</v>
       </c>
       <c r="D10" s="6" t="s">
@@ -3859,7 +4291,7 @@
       <c r="E10" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>50</v>
       </c>
       <c r="G10" t="b">
@@ -3879,16 +4311,16 @@
       <c r="B11" t="s">
         <v>183</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>184</v>
       </c>
       <c r="D11" t="s">
         <v>185</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="12" t="s">
         <v>50</v>
       </c>
       <c r="G11" t="b">
@@ -3908,14 +4340,14 @@
       <c r="B12" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="26" t="s">
         <v>189</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>190</v>
       </c>
       <c r="E12" s="7"/>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="27" t="s">
         <v>50</v>
       </c>
       <c r="G12" s="7" t="b">
@@ -3944,7 +4376,7 @@
       <c r="E13" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="12" t="s">
         <v>50</v>
       </c>
       <c r="G13" t="b">
@@ -3964,14 +4396,14 @@
       <c r="B14" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="28" t="s">
         <v>198</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>199</v>
       </c>
       <c r="E14" s="8"/>
-      <c r="F14" s="28" t="s">
+      <c r="F14" s="27" t="s">
         <v>50</v>
       </c>
       <c r="G14" s="7" t="b">
@@ -3982,157 +4414,161 @@
       </c>
       <c r="I14" s="7"/>
     </row>
-    <row r="15" spans="1:9" ht="27.6">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:9" ht="30">
+      <c r="A15" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="29" t="s">
         <v>200</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="31" t="s">
+      <c r="D15" s="10"/>
+      <c r="E15" s="30" t="s">
         <v>201</v>
       </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-    </row>
-    <row r="16" spans="1:9" ht="27.6">
-      <c r="A16" s="10" t="s">
+      <c r="F15" s="31"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+    </row>
+    <row r="16" spans="1:9" ht="30">
+      <c r="A16" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="31" t="s">
+      <c r="D16" s="10"/>
+      <c r="E16" s="30" t="s">
         <v>204</v>
       </c>
-      <c r="F16" s="32"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="32" t="s">
         <v>145</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="29" t="s">
         <v>206</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="31" t="s">
+      <c r="D17" s="10"/>
+      <c r="E17" s="30" t="s">
         <v>207</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1">
-      <c r="A18" s="34" t="s">
+      <c r="A18" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="60" t="s">
         <v>208</v>
       </c>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="31" t="s">
+      <c r="D18" s="10"/>
+      <c r="E18" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="F18" s="32"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-    </row>
-    <row r="19" spans="1:9" ht="27.6">
-      <c r="A19" s="34" t="s">
+      <c r="F18" s="31"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+    </row>
+    <row r="19" spans="1:9" ht="30">
+      <c r="A19" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="34" t="s">
         <v>212</v>
       </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="31" t="s">
+      <c r="D19" s="10"/>
+      <c r="E19" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="34" t="s">
+      <c r="F19" s="62" t="s">
+        <v>392</v>
+      </c>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+    </row>
+    <row r="20" spans="1:9" ht="30">
+      <c r="A20" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="60" t="s">
         <v>214</v>
       </c>
-      <c r="C20" s="35" t="s">
+      <c r="C20" s="34" t="s">
         <v>215</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="31" t="s">
+      <c r="D20" s="10"/>
+      <c r="E20" s="30" t="s">
         <v>216</v>
       </c>
-      <c r="F20" s="32"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
     </row>
     <row r="21" spans="1:9" ht="13.5" customHeight="1">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="60" t="s">
         <v>188</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="29" t="s">
         <v>217</v>
       </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="31" t="s">
+      <c r="D21" s="10"/>
+      <c r="E21" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-    </row>
-    <row r="22" spans="1:9" ht="27.6">
-      <c r="A22" s="10" t="s">
+      <c r="F21" s="61" t="s">
+        <v>391</v>
+      </c>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+    </row>
+    <row r="22" spans="1:9" ht="30">
+      <c r="A22" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>220</v>
       </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="31" t="s">
+      <c r="D22" s="10"/>
+      <c r="E22" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
@@ -4175,52 +4611,52 @@
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="20"/>
+      <c r="A34" s="19"/>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="36"/>
+      <c r="A35" s="35"/>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="36"/>
+      <c r="A36" s="35"/>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" s="37"/>
+      <c r="A37" s="36"/>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="38"/>
+      <c r="A38" s="37"/>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="36"/>
+      <c r="A39" s="35"/>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" s="36"/>
+      <c r="A40" s="35"/>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" s="37"/>
+      <c r="A41" s="36"/>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="38"/>
+      <c r="A42" s="37"/>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" s="36"/>
+      <c r="A43" s="35"/>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" s="36"/>
+      <c r="A44" s="35"/>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" s="37"/>
+      <c r="A45" s="36"/>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" s="38"/>
+      <c r="A46" s="37"/>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" s="36"/>
+      <c r="A47" s="35"/>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="36"/>
+      <c r="A48" s="35"/>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="37"/>
+      <c r="A49" s="36"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4248,11 +4684,11 @@
     <hyperlink ref="E22" r:id="rId22" xr:uid="{00000000-0004-0000-0100-000015000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <legacyDrawing r:id="rId23"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
+  <legacyDrawing r:id="rId24"/>
   <tableParts count="2">
-    <tablePart r:id="rId24"/>
     <tablePart r:id="rId25"/>
+    <tablePart r:id="rId26"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4260,15 +4696,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I46"/>
-  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="82.3984375" customWidth="1"/>
+    <col min="3" max="3" width="82.42578125" customWidth="1"/>
     <col min="4" max="4" width="45" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="54.296875" customWidth="1"/>
-    <col min="9" max="9" width="109.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.28515625" customWidth="1"/>
+    <col min="9" max="9" width="109.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -4308,14 +4744,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.8">
+    <row r="3" spans="1:9" ht="16.5">
       <c r="A3" s="7" t="s">
         <v>231</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="38" t="s">
         <v>233</v>
       </c>
       <c r="D3" s="7" t="s">
@@ -4337,14 +4773,14 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.8">
+    <row r="4" spans="1:9" ht="16.5">
       <c r="A4" s="7" t="s">
         <v>231</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="38" t="s">
         <v>239</v>
       </c>
       <c r="D4" s="7" t="s">
@@ -4391,7 +4827,7 @@
       </c>
       <c r="I5" s="7"/>
     </row>
-    <row r="6" spans="1:9" ht="70.8">
+    <row r="6" spans="1:9" ht="90.75">
       <c r="A6" t="s">
         <v>231</v>
       </c>
@@ -4404,7 +4840,7 @@
       <c r="D6" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="39" t="s">
         <v>249</v>
       </c>
       <c r="G6" t="b">
@@ -4414,21 +4850,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.8">
+    <row r="7" spans="1:9" ht="16.5">
       <c r="A7" s="7" t="s">
         <v>231</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="38" t="s">
         <v>251</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>252</v>
       </c>
       <c r="E7" s="7"/>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="40" t="s">
         <v>253</v>
       </c>
       <c r="G7" t="b">
@@ -4437,25 +4873,25 @@
       <c r="H7" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="I7" s="40" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16.8">
+    <row r="8" spans="1:9" ht="16.5">
       <c r="A8" s="7" t="s">
         <v>231</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="38" t="s">
         <v>256</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>257</v>
       </c>
       <c r="E8" s="7"/>
-      <c r="F8" s="41" t="s">
+      <c r="F8" s="40" t="s">
         <v>253</v>
       </c>
       <c r="G8" t="b">
@@ -4464,11 +4900,11 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="41" t="s">
+      <c r="I8" s="40" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16.8">
+    <row r="9" spans="1:9" ht="16.5">
       <c r="A9" t="s">
         <v>231</v>
       </c>
@@ -4498,121 +4934,121 @@
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="29" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10" t="s">
+      <c r="D10" s="9"/>
+      <c r="E10" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="F10" s="30"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="30"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="10" t="s">
+      <c r="F10" s="29"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="29"/>
+    </row>
+    <row r="11" spans="1:9" ht="30">
+      <c r="A11" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="29" t="s">
         <v>267</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10" t="s">
+      <c r="D11" s="9"/>
+      <c r="E11" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="F11" s="30"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="30"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="10" t="s">
+      <c r="F11" s="29"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" spans="1:9" ht="30">
+      <c r="A12" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="29" t="s">
         <v>270</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10" t="s">
+      <c r="D12" s="9"/>
+      <c r="E12" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="F12" s="30"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="30"/>
-    </row>
-    <row r="13" spans="1:9" ht="41.4">
-      <c r="A13" s="10" t="s">
+      <c r="F12" s="29"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="29"/>
+    </row>
+    <row r="13" spans="1:9" ht="45">
+      <c r="A13" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>273</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10" t="s">
+      <c r="D13" s="9"/>
+      <c r="E13" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="F13" s="30"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="30"/>
-    </row>
-    <row r="14" spans="1:9" ht="27.6">
-      <c r="A14" s="10" t="s">
+      <c r="F13" s="29"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="29"/>
+    </row>
+    <row r="14" spans="1:9" ht="30">
+      <c r="A14" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>276</v>
       </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10" t="s">
+      <c r="D14" s="9"/>
+      <c r="E14" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="F14" s="30"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="30"/>
-    </row>
-    <row r="15" spans="1:9" ht="16.8">
+      <c r="F14" s="29"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="29"/>
+    </row>
+    <row r="15" spans="1:9" ht="16.5">
       <c r="C15" s="1"/>
       <c r="D15" s="6"/>
-      <c r="E15" s="42"/>
-    </row>
-    <row r="16" spans="1:9" s="3" customFormat="1" ht="16.8">
-      <c r="A16" s="43" t="s">
+      <c r="E15" s="41"/>
+    </row>
+    <row r="16" spans="1:9" s="3" customFormat="1" ht="16.5">
+      <c r="A16" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C16" s="44" t="s">
+      <c r="C16" s="43" t="s">
         <v>259</v>
       </c>
-      <c r="D16" s="45" t="s">
+      <c r="D16" s="44" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="46" t="s">
+      <c r="A17" s="45" t="s">
         <v>231</v>
       </c>
       <c r="B17" t="s">
@@ -4620,7 +5056,7 @@
       </c>
     </row>
     <row r="18" spans="1:2" s="3" customFormat="1">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -4628,7 +5064,7 @@
       </c>
     </row>
     <row r="19" spans="1:2" s="3" customFormat="1">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -4636,7 +5072,7 @@
       </c>
     </row>
     <row r="20" spans="1:2" s="3" customFormat="1">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -4644,7 +5080,7 @@
       </c>
     </row>
     <row r="21" spans="1:2" s="3" customFormat="1">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -4652,7 +5088,7 @@
       </c>
     </row>
     <row r="22" spans="1:2" s="3" customFormat="1">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B22" s="3" t="s">
@@ -4660,23 +5096,23 @@
       </c>
     </row>
     <row r="23" spans="1:2" s="3" customFormat="1">
-      <c r="A23" s="43" t="s">
+      <c r="A23" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="47" customFormat="1">
-      <c r="A24" s="48" t="s">
+    <row r="24" spans="1:2" s="46" customFormat="1">
+      <c r="A24" s="47" t="s">
         <v>231</v>
       </c>
-      <c r="B24" s="47" t="s">
+      <c r="B24" s="46" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="25" spans="1:2" s="3" customFormat="1">
-      <c r="A25" s="43" t="s">
+      <c r="A25" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B25" s="3" t="s">
@@ -4684,7 +5120,7 @@
       </c>
     </row>
     <row r="26" spans="1:2" s="3" customFormat="1">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B26" s="3" t="s">
@@ -4692,7 +5128,7 @@
       </c>
     </row>
     <row r="27" spans="1:2" s="3" customFormat="1">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="42" t="s">
         <v>231</v>
       </c>
       <c r="B27" s="3" t="s">
@@ -4700,10 +5136,10 @@
       </c>
     </row>
     <row r="28" spans="1:2" s="3" customFormat="1">
-      <c r="A28" s="43"/>
+      <c r="A28" s="42"/>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="46"/>
+      <c r="A29" s="45"/>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
@@ -4806,17 +5242,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I34"/>
-  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.8984375" customWidth="1"/>
-    <col min="2" max="2" width="41.59765625" customWidth="1"/>
-    <col min="3" max="3" width="100.8984375" customWidth="1"/>
-    <col min="4" max="4" width="73.69921875" customWidth="1"/>
+    <col min="1" max="1" width="28.85546875" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" customWidth="1"/>
+    <col min="3" max="3" width="100.85546875" customWidth="1"/>
+    <col min="4" max="4" width="73.7109375" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="38.8984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.69921875" customWidth="1"/>
-    <col min="8" max="8" width="19.59765625" customWidth="1"/>
-    <col min="9" max="9" width="57.59765625" customWidth="1"/>
+    <col min="6" max="6" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="57.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -4856,7 +5292,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.8">
+    <row r="3" spans="1:9" ht="16.5">
       <c r="A3" t="s">
         <v>296</v>
       </c>
@@ -4885,7 +5321,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.8">
+    <row r="4" spans="1:9" ht="16.5">
       <c r="A4" t="s">
         <v>296</v>
       </c>
@@ -4930,7 +5366,7 @@
       <c r="F6" t="s">
         <v>306</v>
       </c>
-      <c r="G6" s="49" t="b">
+      <c r="G6" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="b">
@@ -4953,7 +5389,7 @@
       <c r="F7" t="s">
         <v>306</v>
       </c>
-      <c r="G7" s="49" t="b">
+      <c r="G7" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H7" t="b">
@@ -4976,7 +5412,7 @@
       <c r="F8" t="s">
         <v>306</v>
       </c>
-      <c r="G8" s="49" t="b">
+      <c r="G8" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H8" t="b">
@@ -4999,7 +5435,7 @@
       <c r="F9" t="s">
         <v>306</v>
       </c>
-      <c r="G9" s="49" t="b">
+      <c r="G9" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H9" t="b">
@@ -5022,7 +5458,7 @@
       <c r="F10" t="s">
         <v>306</v>
       </c>
-      <c r="G10" s="49" t="b">
+      <c r="G10" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H10" t="b">
@@ -5045,7 +5481,7 @@
       <c r="F11" t="s">
         <v>306</v>
       </c>
-      <c r="G11" s="49" t="b">
+      <c r="G11" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H11" t="b">
@@ -5068,7 +5504,7 @@
       <c r="F12" t="s">
         <v>306</v>
       </c>
-      <c r="G12" s="49" t="b">
+      <c r="G12" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="b">
@@ -5091,7 +5527,7 @@
       <c r="F13" t="s">
         <v>306</v>
       </c>
-      <c r="G13" s="49" t="b">
+      <c r="G13" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H13" t="b">
@@ -5111,7 +5547,7 @@
       <c r="F14" t="s">
         <v>306</v>
       </c>
-      <c r="G14" s="49" t="b">
+      <c r="G14" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H14" t="b">
@@ -5134,7 +5570,7 @@
       <c r="F15" t="s">
         <v>306</v>
       </c>
-      <c r="G15" s="49" t="b">
+      <c r="G15" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H15" t="b">
@@ -5154,13 +5590,13 @@
       <c r="C18" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="11" t="s">
         <v>335</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G18" s="50" t="b">
+      <c r="G18" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H18" s="3" t="b">
@@ -5177,13 +5613,13 @@
       <c r="C19" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="11" t="s">
         <v>335</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G19" s="50" t="b">
+      <c r="G19" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H19" s="3" t="b">
@@ -5200,13 +5636,13 @@
       <c r="C20" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="11" t="s">
         <v>340</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G20" s="50" t="b">
+      <c r="G20" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H20" s="3" t="b">
@@ -5223,13 +5659,13 @@
       <c r="C21" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="11" t="s">
         <v>340</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G21" s="50" t="b">
+      <c r="G21" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H21" s="3" t="b">
@@ -5246,13 +5682,13 @@
       <c r="C22" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="11" t="s">
         <v>345</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G22" s="50" t="b">
+      <c r="G22" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H22" s="3" t="b">
@@ -5269,13 +5705,13 @@
       <c r="C23" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="11" t="s">
         <v>348</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G23" s="50" t="b">
+      <c r="G23" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H23" s="3" t="b">
@@ -5298,7 +5734,7 @@
       <c r="F24" t="s">
         <v>306</v>
       </c>
-      <c r="G24" s="49" t="b">
+      <c r="G24" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H24" t="b">
@@ -5321,7 +5757,7 @@
       <c r="F25" t="s">
         <v>306</v>
       </c>
-      <c r="G25" s="49" t="b">
+      <c r="G25" s="48" t="b">
         <v>1</v>
       </c>
       <c r="H25" t="b">
@@ -5335,7 +5771,7 @@
       <c r="B26" s="7" t="s">
         <v>355</v>
       </c>
-      <c r="C26" s="51" t="s">
+      <c r="C26" s="50" t="s">
         <v>356</v>
       </c>
       <c r="E26" s="2" t="s">
@@ -5346,23 +5782,23 @@
       </c>
     </row>
     <row r="28" spans="1:8" s="3" customFormat="1">
-      <c r="A28" s="52" t="s">
+      <c r="A28" s="51" t="s">
         <v>296</v>
       </c>
-      <c r="B28" s="53" t="s">
+      <c r="B28" s="52" t="s">
         <v>358</v>
       </c>
-      <c r="C28" s="54" t="s">
+      <c r="C28" s="53" t="s">
         <v>359</v>
       </c>
-      <c r="D28" s="52"/>
-      <c r="E28" s="55" t="s">
+      <c r="D28" s="51"/>
+      <c r="E28" s="54" t="s">
         <v>360</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G28" s="50" t="b">
+      <c r="G28" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H28" s="3" t="b">
@@ -5370,23 +5806,23 @@
       </c>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="52" t="s">
+      <c r="A29" s="51" t="s">
         <v>296</v>
       </c>
-      <c r="B29" s="53" t="s">
+      <c r="B29" s="52" t="s">
         <v>361</v>
       </c>
-      <c r="C29" s="54" t="s">
+      <c r="C29" s="53" t="s">
         <v>362</v>
       </c>
       <c r="D29" s="3"/>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="11" t="s">
         <v>363</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G29" s="50" t="b">
+      <c r="G29" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H29" s="3" t="b">
@@ -5394,23 +5830,23 @@
       </c>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="51" t="s">
         <v>296</v>
       </c>
-      <c r="B30" s="53" t="s">
+      <c r="B30" s="52" t="s">
         <v>364</v>
       </c>
-      <c r="C30" s="54" t="s">
+      <c r="C30" s="53" t="s">
         <v>365</v>
       </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="12" t="s">
+      <c r="E30" s="11" t="s">
         <v>366</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G30" s="50" t="b">
+      <c r="G30" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H30" s="3" t="b">
@@ -5418,23 +5854,23 @@
       </c>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="52" t="s">
+      <c r="A31" s="51" t="s">
         <v>296</v>
       </c>
-      <c r="B31" s="56" t="s">
+      <c r="B31" s="55" t="s">
         <v>341</v>
       </c>
-      <c r="C31" s="54" t="s">
+      <c r="C31" s="53" t="s">
         <v>367</v>
       </c>
       <c r="D31" s="3"/>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="11" t="s">
         <v>368</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G31" s="50" t="b">
+      <c r="G31" s="49" t="b">
         <v>1</v>
       </c>
       <c r="H31" s="3" t="b">
@@ -5450,7 +5886,7 @@
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="56" t="s">
         <v>369</v>
       </c>
       <c r="B34" t="s">
@@ -5498,13 +5934,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="50.69921875" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="82.09765625" customWidth="1"/>
-    <col min="4" max="4" width="110" customWidth="1"/>
-    <col min="5" max="9" width="50.69921875" customWidth="1"/>
+    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="66.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="6.85546875" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" customWidth="1"/>
+    <col min="8" max="8" width="6" customWidth="1"/>
+    <col min="9" max="9" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -5548,106 +5988,173 @@
       <c r="A3" t="s">
         <v>372</v>
       </c>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="57" t="s">
         <v>373</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="60" t="s">
         <v>374</v>
+      </c>
+      <c r="D3" t="s">
+        <v>393</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>372</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="57" t="s">
         <v>375</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="60" t="s">
         <v>376</v>
+      </c>
+      <c r="D4" s="66" t="s">
+        <v>397</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>372</v>
       </c>
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="57" t="s">
         <v>377</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="60" t="s">
         <v>378</v>
       </c>
       <c r="F5" t="s">
         <v>306</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>372</v>
       </c>
-      <c r="B6" s="58" t="s">
+      <c r="B6" s="57" t="s">
         <v>379</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="60" t="s">
         <v>380</v>
       </c>
       <c r="F6" t="s">
         <v>306</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>372</v>
       </c>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="57" t="s">
         <v>381</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="60" t="s">
         <v>382</v>
       </c>
       <c r="F7" t="s">
         <v>306</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>372</v>
       </c>
-      <c r="B8" s="54" t="s">
+      <c r="B8" s="53" t="s">
         <v>383</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="66" t="s">
         <v>384</v>
       </c>
       <c r="F8" t="s">
         <v>306</v>
+      </c>
+      <c r="I8" s="66" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>372</v>
       </c>
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="53" t="s">
         <v>385</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="66" t="s">
         <v>386</v>
       </c>
       <c r="F9" t="s">
         <v>306</v>
+      </c>
+      <c r="I9" s="66" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>372</v>
       </c>
-      <c r="B10" s="54" t="s">
+      <c r="B10" s="53" t="s">
         <v>387</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="66" t="s">
         <v>388</v>
       </c>
       <c r="F10" t="s">
         <v>306</v>
+      </c>
+      <c r="I10" s="66" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="B11" s="65" t="s">
+        <v>394</v>
+      </c>
+      <c r="C11" s="66" t="s">
+        <v>395</v>
+      </c>
+      <c r="D11" t="s">
+        <v>396</v>
+      </c>
+      <c r="I11" s="66" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>390</v>
+      </c>
+      <c r="B14" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -5659,7 +6166,7 @@
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="56" t="s">
         <v>369</v>
       </c>
       <c r="B18" t="s">
@@ -5677,4 +6184,215 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCB2661C-F7D3-454D-BA5E-50A399AE0093}">
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="52.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="67" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="67" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="67" t="s">
+        <v>230</v>
+      </c>
+      <c r="E2" s="67" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="67" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="67" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="63" t="s">
+        <v>398</v>
+      </c>
+      <c r="B3" s="68" t="s">
+        <v>411</v>
+      </c>
+      <c r="C3" s="63" t="s">
+        <v>412</v>
+      </c>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63" t="s">
+        <v>413</v>
+      </c>
+      <c r="F3" s="63"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="64" t="s">
+        <v>399</v>
+      </c>
+      <c r="B4" s="64" t="s">
+        <v>418</v>
+      </c>
+      <c r="C4" s="64" t="s">
+        <v>417</v>
+      </c>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="63" t="s">
+        <v>400</v>
+      </c>
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="70" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="64" t="s">
+        <v>401</v>
+      </c>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="F6" s="64"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="63" t="s">
+        <v>402</v>
+      </c>
+      <c r="B7" s="63"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="64" t="s">
+        <v>403</v>
+      </c>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="F8" s="64"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="63" t="s">
+        <v>404</v>
+      </c>
+      <c r="B9" s="63"/>
+      <c r="C9" s="63"/>
+      <c r="D9" s="63"/>
+      <c r="E9" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="F9" s="63"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="64" t="s">
+        <v>405</v>
+      </c>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="F10" s="64"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="63" t="s">
+        <v>406</v>
+      </c>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="64" t="s">
+        <v>413</v>
+      </c>
+      <c r="F11" s="63"/>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="66" t="s">
+        <v>419</v>
+      </c>
+      <c r="B17" s="66" t="s">
+        <v>423</v>
+      </c>
+      <c r="C17" s="66" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="409.5">
+      <c r="A18" s="69" t="s">
+        <v>420</v>
+      </c>
+      <c r="B18" s="69" t="s">
+        <v>422</v>
+      </c>
+      <c r="C18" s="69" t="s">
+        <v>424</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" display="https://taskman.eionet.europa.eu/issues/306644" xr:uid="{C17BE7F8-96E2-4B24-B3C1-A2C6C1077CEC}"/>
+    <hyperlink ref="A4" r:id="rId2" display="https://taskman.eionet.europa.eu/issues/306645" xr:uid="{669798E4-CA87-46A3-8FF3-548FFD412461}"/>
+    <hyperlink ref="A5" r:id="rId3" display="https://taskman.eionet.europa.eu/issues/306646" xr:uid="{600BAD42-B19C-4FB6-8778-ACC50F68FECE}"/>
+    <hyperlink ref="A6" r:id="rId4" display="https://taskman.eionet.europa.eu/issues/306647" xr:uid="{D31DFE2A-2C13-4490-92A4-F015EB6482DE}"/>
+    <hyperlink ref="A7" r:id="rId5" display="https://taskman.eionet.europa.eu/issues/306648" xr:uid="{A7EAC514-95A7-4B56-A1AE-2C2B2E83F7FA}"/>
+    <hyperlink ref="A8" r:id="rId6" display="https://taskman.eionet.europa.eu/issues/306649" xr:uid="{725BE1C0-8AC3-4D1A-8B5A-DED0A1449587}"/>
+    <hyperlink ref="A9" r:id="rId7" display="https://taskman.eionet.europa.eu/issues/306650" xr:uid="{24DF69DC-3794-4A8D-8B6B-B55423B4C424}"/>
+    <hyperlink ref="A10" r:id="rId8" display="https://taskman.eionet.europa.eu/issues/306651" xr:uid="{BF3C2CC0-50FD-49AB-A76A-3871EF2AAEEA}"/>
+    <hyperlink ref="A11" r:id="rId9" display="https://taskman.eionet.europa.eu/issues/306652" xr:uid="{FAC06DF6-8FD9-40C9-BF23-E0019C3F4728}"/>
+    <hyperlink ref="A12" r:id="rId10" display="https://taskman.eionet.europa.eu/issues/306653" xr:uid="{4B78FB83-4BEB-4109-82DB-96D9DF55C7A8}"/>
+    <hyperlink ref="A13" r:id="rId11" display="https://taskman.eionet.europa.eu/issues/306654" xr:uid="{99D6138B-3DFA-405F-8A45-95BFA4F992D8}"/>
+    <hyperlink ref="A14" r:id="rId12" display="https://taskman.eionet.europa.eu/issues/306655" xr:uid="{228B36E5-77B5-4A60-A9EC-BC8B21292E79}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId13"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update AQD R3 DDBB views 2026_4sfera_com.xlsx
Update of the excel
</commit_message>
<xml_diff>
--- a/AQD R3 DDBB views 2026_4sfera_com.xlsx
+++ b/AQD R3 DDBB views 2026_4sfera_com.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYECTOS\AQD migration to R3\github\AirQualityInReportNet3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1442F60B-5818-4D61-96E1-7B9AEE7D21CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A021E6B8-AB2F-4CA8-9116-7169803714E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="1692" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SamplingProcess (SPP)" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="SamplingPoint (SPO)" sheetId="3" r:id="rId3"/>
     <sheet name="SamplingPointLocation (SPL) " sheetId="4" r:id="rId4"/>
     <sheet name="ZoneGeometry (ZOG)" sheetId="5" r:id="rId5"/>
-    <sheet name="Authority (AUT)" sheetId="6" r:id="rId6"/>
+    <sheet name="NOT READY Authority (AUT)" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -241,7 +241,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="427">
   <si>
     <t>2026 task</t>
   </si>
@@ -2023,16 +2023,26 @@
   <si>
     <t>test AUT_04</t>
   </si>
+  <si>
+    <t xml:space="preserve">NOT READY </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2372,102 +2382,103 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2476,6 +2487,28 @@
     <cellStyle name="Normal 2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
   <dxfs count="16">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFDD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2499,28 +2532,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFDD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -2701,10 +2712,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0BC4E8C3-85C6-489D-BF2D-740644FE565C}" name="Table11" displayName="Table11" ref="A2:G14" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0BC4E8C3-85C6-489D-BF2D-740644FE565C}" name="Table11" displayName="Table11" ref="A2:G14" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1">
   <autoFilter ref="A2:G14" xr:uid="{0BC4E8C3-85C6-489D-BF2D-740644FE565C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{FCB4B3CE-80E1-443E-8E4E-D4DAF8DBF592}" name="QC rule" dataDxfId="1" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{FCB4B3CE-80E1-443E-8E4E-D4DAF8DBF592}" name="QC rule" dataDxfId="0" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{F270D045-3F54-41FB-B521-15F84117A486}" name="Description"/>
     <tableColumn id="3" xr3:uid="{9F2AADD6-BEE8-40A8-983C-2459092F782C}" name="Task"/>
     <tableColumn id="4" xr3:uid="{A35617F8-F712-4679-B5D7-2B7086D1C24B}" name="Task 2"/>
@@ -3143,7 +3154,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I51"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -3155,7 +3166,7 @@
     <col min="9" max="9" width="71.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3163,7 +3174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -3192,7 +3203,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5">
+    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3215,7 +3226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -3241,7 +3252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -3267,7 +3278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -3293,7 +3304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="3" customFormat="1">
+    <row r="7" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -3316,7 +3327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="3" customFormat="1">
+    <row r="8" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
@@ -3339,7 +3350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="3" customFormat="1">
+    <row r="9" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -3362,7 +3373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -3388,7 +3399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -3414,7 +3425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -3440,7 +3451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -3466,7 +3477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -3492,7 +3503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -3518,7 +3529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -3544,7 +3555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -3573,7 +3584,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -3602,7 +3613,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -3628,7 +3639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -3654,7 +3665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>11</v>
       </c>
@@ -3678,7 +3689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="3" customFormat="1">
+    <row r="22" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>11</v>
       </c>
@@ -3701,7 +3712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>11</v>
       </c>
@@ -3725,7 +3736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>11</v>
       </c>
@@ -3749,7 +3760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>11</v>
       </c>
@@ -3764,7 +3775,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75">
+    <row r="26" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>11</v>
       </c>
@@ -3779,7 +3790,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>11</v>
       </c>
@@ -3794,7 +3805,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="58" customFormat="1">
+    <row r="28" spans="1:9" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="58" t="s">
         <v>11</v>
       </c>
@@ -3808,7 +3819,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="58" customFormat="1">
+    <row r="29" spans="1:9" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="58" t="s">
         <v>11</v>
       </c>
@@ -3822,7 +3833,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="58" customFormat="1">
+    <row r="30" spans="1:9" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="58" t="s">
         <v>11</v>
       </c>
@@ -3836,7 +3847,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="58" customFormat="1">
+    <row r="31" spans="1:9" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="58" t="s">
         <v>11</v>
       </c>
@@ -3850,7 +3861,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="58" customFormat="1">
+    <row r="32" spans="1:9" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="58" t="s">
         <v>11</v>
       </c>
@@ -3864,7 +3875,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="58" customFormat="1">
+    <row r="33" spans="1:5" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="58" t="s">
         <v>11</v>
       </c>
@@ -3878,7 +3889,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>124</v>
       </c>
@@ -3886,7 +3897,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>126</v>
       </c>
@@ -3894,7 +3905,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>128</v>
       </c>
@@ -3902,7 +3913,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>130</v>
       </c>
@@ -3910,7 +3921,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>131</v>
       </c>
@@ -3918,7 +3929,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>132</v>
       </c>
@@ -3926,19 +3937,19 @@
         <v>133</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>135</v>
       </c>
       <c r="D42" s="12"/>
       <c r="E42" s="12"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>136</v>
       </c>
@@ -3946,7 +3957,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>138</v>
       </c>
@@ -3954,15 +3965,15 @@
         <v>139</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="13"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
         <v>63</v>
       </c>
@@ -3970,7 +3981,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
         <v>108</v>
       </c>
@@ -3981,7 +3992,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>95</v>
       </c>
@@ -3992,7 +4003,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
         <v>98</v>
       </c>
@@ -4043,7 +4054,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.140625" customWidth="1"/>
@@ -4055,7 +4066,7 @@
     <col min="9" max="9" width="185.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4063,7 +4074,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4092,7 +4103,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1">
+    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>145</v>
       </c>
@@ -4121,7 +4132,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>145</v>
       </c>
@@ -4147,7 +4158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>145</v>
       </c>
@@ -4173,7 +4184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="22" customFormat="1">
+    <row r="6" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
         <v>145</v>
       </c>
@@ -4196,7 +4207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="24" customFormat="1">
+    <row r="7" spans="1:9" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
         <v>145</v>
       </c>
@@ -4223,7 +4234,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>145</v>
       </c>
@@ -4249,7 +4260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>145</v>
       </c>
@@ -4275,7 +4286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>145</v>
       </c>
@@ -4304,7 +4315,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>145</v>
       </c>
@@ -4333,7 +4344,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>145</v>
       </c>
@@ -4360,7 +4371,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>145</v>
       </c>
@@ -4389,7 +4400,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>145</v>
       </c>
@@ -4414,7 +4425,7 @@
       </c>
       <c r="I14" s="7"/>
     </row>
-    <row r="15" spans="1:9" ht="30">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>145</v>
       </c>
@@ -4433,7 +4444,7 @@
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:9" ht="30">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>145</v>
       </c>
@@ -4452,7 +4463,7 @@
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="32" t="s">
         <v>145</v>
       </c>
@@ -4471,7 +4482,7 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="1:9" ht="18" customHeight="1">
+    <row r="18" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
         <v>145</v>
       </c>
@@ -4490,7 +4501,7 @@
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="1:9" ht="30">
+    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
         <v>145</v>
       </c>
@@ -4511,7 +4522,7 @@
       <c r="H19" s="9"/>
       <c r="I19" s="9"/>
     </row>
-    <row r="20" spans="1:9" ht="30">
+    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
         <v>145</v>
       </c>
@@ -4530,7 +4541,7 @@
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
     </row>
-    <row r="21" spans="1:9" ht="13.5" customHeight="1">
+    <row r="21" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>145</v>
       </c>
@@ -4551,7 +4562,7 @@
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
     </row>
-    <row r="22" spans="1:9" ht="30">
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>145</v>
       </c>
@@ -4570,7 +4581,7 @@
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>124</v>
       </c>
@@ -4578,7 +4589,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>222</v>
       </c>
@@ -4586,7 +4597,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>224</v>
       </c>
@@ -4594,7 +4605,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>132</v>
       </c>
@@ -4602,7 +4613,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>227</v>
       </c>
@@ -4610,52 +4621,52 @@
         <v>228</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="19"/>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="35"/>
     </row>
-    <row r="36" spans="1:1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="35"/>
     </row>
-    <row r="37" spans="1:1">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="36"/>
     </row>
-    <row r="38" spans="1:1">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="37"/>
     </row>
-    <row r="39" spans="1:1">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="35"/>
     </row>
-    <row r="40" spans="1:1">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="35"/>
     </row>
-    <row r="41" spans="1:1">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="36"/>
     </row>
-    <row r="42" spans="1:1">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="37"/>
     </row>
-    <row r="43" spans="1:1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="35"/>
     </row>
-    <row r="44" spans="1:1">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="35"/>
     </row>
-    <row r="45" spans="1:1">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="36"/>
     </row>
-    <row r="46" spans="1:1">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="37"/>
     </row>
-    <row r="47" spans="1:1">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="35"/>
     </row>
-    <row r="48" spans="1:1">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="35"/>
     </row>
-    <row r="49" spans="1:1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="36"/>
     </row>
   </sheetData>
@@ -4696,7 +4707,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I46"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
@@ -4707,7 +4718,7 @@
     <col min="9" max="9" width="109.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4715,7 +4726,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4744,7 +4755,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5">
+    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>231</v>
       </c>
@@ -4773,7 +4784,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5">
+    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>231</v>
       </c>
@@ -4800,7 +4811,7 @@
       </c>
       <c r="I4" s="7"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>231</v>
       </c>
@@ -4827,7 +4838,7 @@
       </c>
       <c r="I5" s="7"/>
     </row>
-    <row r="6" spans="1:9" ht="90.75">
+    <row r="6" spans="1:9" ht="90.75" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>231</v>
       </c>
@@ -4850,7 +4861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.5">
+    <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>231</v>
       </c>
@@ -4877,7 +4888,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16.5">
+    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>231</v>
       </c>
@@ -4904,7 +4915,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16.5">
+    <row r="9" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>231</v>
       </c>
@@ -4933,7 +4944,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>231</v>
       </c>
@@ -4952,7 +4963,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="29"/>
     </row>
-    <row r="11" spans="1:9" ht="30">
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>231</v>
       </c>
@@ -4971,7 +4982,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="29"/>
     </row>
-    <row r="12" spans="1:9" ht="30">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>231</v>
       </c>
@@ -4990,7 +5001,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="29"/>
     </row>
-    <row r="13" spans="1:9" ht="45">
+    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>231</v>
       </c>
@@ -5009,7 +5020,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="29"/>
     </row>
-    <row r="14" spans="1:9" ht="30">
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>231</v>
       </c>
@@ -5028,12 +5039,12 @@
       <c r="H14" s="9"/>
       <c r="I14" s="29"/>
     </row>
-    <row r="15" spans="1:9" ht="16.5">
+    <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="C15" s="1"/>
       <c r="D15" s="6"/>
       <c r="E15" s="41"/>
     </row>
-    <row r="16" spans="1:9" s="3" customFormat="1" ht="16.5">
+    <row r="16" spans="1:9" s="3" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="42" t="s">
         <v>231</v>
       </c>
@@ -5047,7 +5058,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="45" t="s">
         <v>231</v>
       </c>
@@ -5055,7 +5066,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="3" customFormat="1">
+    <row r="18" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="42" t="s">
         <v>231</v>
       </c>
@@ -5063,7 +5074,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="3" customFormat="1">
+    <row r="19" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="42" t="s">
         <v>231</v>
       </c>
@@ -5071,7 +5082,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="20" spans="1:2" s="3" customFormat="1">
+    <row r="20" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="42" t="s">
         <v>231</v>
       </c>
@@ -5079,7 +5090,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="21" spans="1:2" s="3" customFormat="1">
+    <row r="21" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="42" t="s">
         <v>231</v>
       </c>
@@ -5087,7 +5098,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="22" spans="1:2" s="3" customFormat="1">
+    <row r="22" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="42" t="s">
         <v>231</v>
       </c>
@@ -5095,7 +5106,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="23" spans="1:2" s="3" customFormat="1">
+    <row r="23" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="42" t="s">
         <v>231</v>
       </c>
@@ -5103,7 +5114,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="46" customFormat="1">
+    <row r="24" spans="1:2" s="46" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
         <v>231</v>
       </c>
@@ -5111,7 +5122,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="25" spans="1:2" s="3" customFormat="1">
+    <row r="25" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="42" t="s">
         <v>231</v>
       </c>
@@ -5119,7 +5130,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="26" spans="1:2" s="3" customFormat="1">
+    <row r="26" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="42" t="s">
         <v>231</v>
       </c>
@@ -5127,7 +5138,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="27" spans="1:2" s="3" customFormat="1">
+    <row r="27" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="42" t="s">
         <v>231</v>
       </c>
@@ -5135,13 +5146,13 @@
         <v>284</v>
       </c>
     </row>
-    <row r="28" spans="1:2" s="3" customFormat="1">
+    <row r="28" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="42"/>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="45"/>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>124</v>
       </c>
@@ -5149,7 +5160,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>224</v>
       </c>
@@ -5157,7 +5168,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>285</v>
       </c>
@@ -5165,7 +5176,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>132</v>
       </c>
@@ -5173,42 +5184,42 @@
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>294</v>
       </c>
@@ -5242,10 +5253,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.85546875" customWidth="1"/>
-    <col min="2" max="2" width="41.5703125" customWidth="1"/>
+    <col min="2" max="2" width="28.5703125" customWidth="1"/>
     <col min="3" max="3" width="100.85546875" customWidth="1"/>
     <col min="4" max="4" width="73.7109375" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
@@ -5255,7 +5266,7 @@
     <col min="9" max="9" width="57.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5263,7 +5274,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -5292,7 +5303,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5">
+    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>296</v>
       </c>
@@ -5321,7 +5332,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5">
+    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>296</v>
       </c>
@@ -5350,7 +5361,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>296</v>
       </c>
@@ -5373,7 +5384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>296</v>
       </c>
@@ -5396,7 +5407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>296</v>
       </c>
@@ -5419,7 +5430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -5442,7 +5453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>296</v>
       </c>
@@ -5465,7 +5476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>296</v>
       </c>
@@ -5488,7 +5499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>296</v>
       </c>
@@ -5511,7 +5522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>296</v>
       </c>
@@ -5534,7 +5545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>296</v>
       </c>
@@ -5554,7 +5565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>296</v>
       </c>
@@ -5580,7 +5591,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="3" customFormat="1">
+    <row r="18" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>296</v>
       </c>
@@ -5603,7 +5614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="3" customFormat="1">
+    <row r="19" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>296</v>
       </c>
@@ -5626,7 +5637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="3" customFormat="1">
+    <row r="20" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>296</v>
       </c>
@@ -5649,7 +5660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="3" customFormat="1">
+    <row r="21" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>296</v>
       </c>
@@ -5672,7 +5683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="3" customFormat="1">
+    <row r="22" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>296</v>
       </c>
@@ -5695,7 +5706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="3" customFormat="1">
+    <row r="23" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>296</v>
       </c>
@@ -5718,7 +5729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>296</v>
       </c>
@@ -5741,7 +5752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>296</v>
       </c>
@@ -5764,7 +5775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>296</v>
       </c>
@@ -5781,7 +5792,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="3" customFormat="1">
+    <row r="28" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="51" t="s">
         <v>296</v>
       </c>
@@ -5805,7 +5816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="51" t="s">
         <v>296</v>
       </c>
@@ -5829,7 +5840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="51" t="s">
         <v>296</v>
       </c>
@@ -5853,7 +5864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="51" t="s">
         <v>296</v>
       </c>
@@ -5877,7 +5888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>124</v>
       </c>
@@ -5885,7 +5896,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="56" t="s">
         <v>369</v>
       </c>
@@ -5934,11 +5945,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="66.140625" customWidth="1"/>
+    <col min="3" max="3" width="75.5703125" customWidth="1"/>
     <col min="4" max="4" width="17.85546875" customWidth="1"/>
     <col min="5" max="5" width="6.85546875" customWidth="1"/>
     <col min="6" max="6" width="6.7109375" customWidth="1"/>
@@ -5947,7 +5958,7 @@
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5955,7 +5966,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -5984,7 +5995,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>372</v>
       </c>
@@ -6004,7 +6015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>372</v>
       </c>
@@ -6024,7 +6035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>372</v>
       </c>
@@ -6044,7 +6055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>372</v>
       </c>
@@ -6064,7 +6075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>372</v>
       </c>
@@ -6084,14 +6095,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>372</v>
       </c>
       <c r="B8" s="53" t="s">
         <v>383</v>
       </c>
-      <c r="C8" s="66" t="s">
+      <c r="C8" s="71" t="s">
         <v>384</v>
       </c>
       <c r="F8" t="s">
@@ -6101,7 +6112,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>372</v>
       </c>
@@ -6118,14 +6129,14 @@
         <v>416</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>372</v>
       </c>
       <c r="B10" s="53" t="s">
         <v>387</v>
       </c>
-      <c r="C10" s="66" t="s">
+      <c r="C10" s="71" t="s">
         <v>388</v>
       </c>
       <c r="F10" t="s">
@@ -6135,11 +6146,14 @@
         <v>414</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>372</v>
+      </c>
       <c r="B11" s="65" t="s">
         <v>394</v>
       </c>
-      <c r="C11" s="66" t="s">
+      <c r="C11" s="71" t="s">
         <v>395</v>
       </c>
       <c r="D11" t="s">
@@ -6149,7 +6163,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>390</v>
       </c>
@@ -6157,7 +6171,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>124</v>
       </c>
@@ -6165,7 +6179,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="56" t="s">
         <v>369</v>
       </c>
@@ -6189,20 +6203,23 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCB2661C-F7D3-454D-BA5E-50A399AE0093}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="6" max="6" width="9.28515625" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="B1" s="58" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="67" t="s">
         <v>3</v>
       </c>
@@ -6225,7 +6242,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
         <v>398</v>
       </c>
@@ -6241,7 +6258,7 @@
       </c>
       <c r="F3" s="63"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="64" t="s">
         <v>399</v>
       </c>
@@ -6255,7 +6272,7 @@
       <c r="E4" s="64"/>
       <c r="F4" s="64"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="63" t="s">
         <v>400</v>
       </c>
@@ -6268,7 +6285,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="64" t="s">
         <v>401</v>
       </c>
@@ -6280,7 +6297,7 @@
       </c>
       <c r="F6" s="64"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="63" t="s">
         <v>402</v>
       </c>
@@ -6290,7 +6307,7 @@
       <c r="E7" s="63"/>
       <c r="F7" s="63"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="64" t="s">
         <v>403</v>
       </c>
@@ -6302,7 +6319,7 @@
       </c>
       <c r="F8" s="64"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="63" t="s">
         <v>404</v>
       </c>
@@ -6314,7 +6331,7 @@
       </c>
       <c r="F9" s="63"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="64" t="s">
         <v>405</v>
       </c>
@@ -6326,7 +6343,7 @@
       </c>
       <c r="F10" s="64"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
         <v>406</v>
       </c>
@@ -6338,22 +6355,22 @@
       </c>
       <c r="F11" s="63"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="66" t="s">
         <v>419</v>
       </c>
@@ -6364,7 +6381,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="409.5">
+    <row r="18" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A18" s="69" t="s">
         <v>420</v>
       </c>

</xml_diff>